<commit_message>
Add manning alerts, role coverage, fairness counters, more statuses
- Six daily statuses (base/home/vacation/medical/course/conditions) via
  dropdown with auto color-coding.
- Daily rows: total at base + armory/quartermaster coverage, turning red
  below editable manning thresholds.
- Per-soldier fairness counters (base/home days, weekends and holidays at
  home) with a color scale to spot imbalance.
- Demo preview image illustrating colors and the red under-manning alert.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/shavtzak_yetziot.xlsx
+++ b/shavtzak_yetziot.xlsx
@@ -48,7 +48,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -77,12 +77,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4A7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF5050"/>
       </patternFill>
     </fill>
   </fills>
@@ -112,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,18 +170,44 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -167,7 +218,28 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00BDD7EE"/>
+          <fgColor rgb="00A9D08E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B4A7D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -533,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CZ26"/>
+  <dimension ref="A1:DB35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -640,6 +712,8 @@
     <col width="5" customWidth="1" min="102" max="102"/>
     <col width="9" customWidth="1" min="103" max="103"/>
     <col width="9" customWidth="1" min="104" max="104"/>
+    <col width="9" customWidth="1" min="105" max="105"/>
+    <col width="9" customWidth="1" min="106" max="106"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1283,12 +1357,22 @@
       </c>
       <c r="CY3" s="2" t="inlineStr">
         <is>
+          <t>ימי בסיס</t>
+        </is>
+      </c>
+      <c r="CZ3" s="2" t="inlineStr">
+        <is>
           <t>ימי בית</t>
         </is>
       </c>
-      <c r="CZ3" s="2" t="inlineStr">
-        <is>
-          <t>ימי בסיס</t>
+      <c r="DA3" s="2" t="inlineStr">
+        <is>
+          <t>סופ"ש בבית</t>
+        </is>
+      </c>
+      <c r="DB3" s="2" t="inlineStr">
+        <is>
+          <t>חגים בבית</t>
         </is>
       </c>
     </row>
@@ -1404,11 +1488,19 @@
       <c r="CW4" s="8" t="n"/>
       <c r="CX4" s="8" t="n"/>
       <c r="CY4" s="9">
+        <f>COUNTIF(D4:CX4,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ4" s="9">
         <f>COUNTIF(D4:CX4,"בית")</f>
         <v/>
       </c>
-      <c r="CZ4" s="9">
-        <f>COUNTIF(D4:CX4,"בסיס")</f>
+      <c r="DA4" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D4:CX4="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB4" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D4:CX4="בית"))</f>
         <v/>
       </c>
     </row>
@@ -1524,11 +1616,19 @@
       <c r="CW5" s="8" t="n"/>
       <c r="CX5" s="8" t="n"/>
       <c r="CY5" s="9">
+        <f>COUNTIF(D5:CX5,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ5" s="9">
         <f>COUNTIF(D5:CX5,"בית")</f>
         <v/>
       </c>
-      <c r="CZ5" s="9">
-        <f>COUNTIF(D5:CX5,"בסיס")</f>
+      <c r="DA5" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D5:CX5="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB5" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D5:CX5="בית"))</f>
         <v/>
       </c>
     </row>
@@ -1644,11 +1744,19 @@
       <c r="CW6" s="8" t="n"/>
       <c r="CX6" s="8" t="n"/>
       <c r="CY6" s="9">
+        <f>COUNTIF(D6:CX6,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ6" s="9">
         <f>COUNTIF(D6:CX6,"בית")</f>
         <v/>
       </c>
-      <c r="CZ6" s="9">
-        <f>COUNTIF(D6:CX6,"בסיס")</f>
+      <c r="DA6" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D6:CX6="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB6" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D6:CX6="בית"))</f>
         <v/>
       </c>
     </row>
@@ -1764,11 +1872,19 @@
       <c r="CW7" s="8" t="n"/>
       <c r="CX7" s="8" t="n"/>
       <c r="CY7" s="9">
+        <f>COUNTIF(D7:CX7,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ7" s="9">
         <f>COUNTIF(D7:CX7,"בית")</f>
         <v/>
       </c>
-      <c r="CZ7" s="9">
-        <f>COUNTIF(D7:CX7,"בסיס")</f>
+      <c r="DA7" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D7:CX7="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB7" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D7:CX7="בית"))</f>
         <v/>
       </c>
     </row>
@@ -1884,11 +2000,19 @@
       <c r="CW8" s="8" t="n"/>
       <c r="CX8" s="8" t="n"/>
       <c r="CY8" s="9">
+        <f>COUNTIF(D8:CX8,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ8" s="9">
         <f>COUNTIF(D8:CX8,"בית")</f>
         <v/>
       </c>
-      <c r="CZ8" s="9">
-        <f>COUNTIF(D8:CX8,"בסיס")</f>
+      <c r="DA8" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D8:CX8="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB8" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D8:CX8="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2004,11 +2128,19 @@
       <c r="CW9" s="8" t="n"/>
       <c r="CX9" s="8" t="n"/>
       <c r="CY9" s="9">
+        <f>COUNTIF(D9:CX9,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ9" s="9">
         <f>COUNTIF(D9:CX9,"בית")</f>
         <v/>
       </c>
-      <c r="CZ9" s="9">
-        <f>COUNTIF(D9:CX9,"בסיס")</f>
+      <c r="DA9" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D9:CX9="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB9" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D9:CX9="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2124,11 +2256,19 @@
       <c r="CW10" s="8" t="n"/>
       <c r="CX10" s="8" t="n"/>
       <c r="CY10" s="9">
+        <f>COUNTIF(D10:CX10,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ10" s="9">
         <f>COUNTIF(D10:CX10,"בית")</f>
         <v/>
       </c>
-      <c r="CZ10" s="9">
-        <f>COUNTIF(D10:CX10,"בסיס")</f>
+      <c r="DA10" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D10:CX10="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB10" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D10:CX10="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2244,11 +2384,19 @@
       <c r="CW11" s="8" t="n"/>
       <c r="CX11" s="8" t="n"/>
       <c r="CY11" s="9">
+        <f>COUNTIF(D11:CX11,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ11" s="9">
         <f>COUNTIF(D11:CX11,"בית")</f>
         <v/>
       </c>
-      <c r="CZ11" s="9">
-        <f>COUNTIF(D11:CX11,"בסיס")</f>
+      <c r="DA11" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D11:CX11="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB11" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D11:CX11="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2364,11 +2512,19 @@
       <c r="CW12" s="8" t="n"/>
       <c r="CX12" s="8" t="n"/>
       <c r="CY12" s="9">
+        <f>COUNTIF(D12:CX12,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ12" s="9">
         <f>COUNTIF(D12:CX12,"בית")</f>
         <v/>
       </c>
-      <c r="CZ12" s="9">
-        <f>COUNTIF(D12:CX12,"בסיס")</f>
+      <c r="DA12" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D12:CX12="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB12" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D12:CX12="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2484,11 +2640,19 @@
       <c r="CW13" s="8" t="n"/>
       <c r="CX13" s="8" t="n"/>
       <c r="CY13" s="9">
+        <f>COUNTIF(D13:CX13,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ13" s="9">
         <f>COUNTIF(D13:CX13,"בית")</f>
         <v/>
       </c>
-      <c r="CZ13" s="9">
-        <f>COUNTIF(D13:CX13,"בסיס")</f>
+      <c r="DA13" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D13:CX13="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB13" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D13:CX13="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2604,11 +2768,19 @@
       <c r="CW14" s="8" t="n"/>
       <c r="CX14" s="8" t="n"/>
       <c r="CY14" s="9">
+        <f>COUNTIF(D14:CX14,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ14" s="9">
         <f>COUNTIF(D14:CX14,"בית")</f>
         <v/>
       </c>
-      <c r="CZ14" s="9">
-        <f>COUNTIF(D14:CX14,"בסיס")</f>
+      <c r="DA14" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D14:CX14="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB14" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D14:CX14="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2724,11 +2896,19 @@
       <c r="CW15" s="8" t="n"/>
       <c r="CX15" s="8" t="n"/>
       <c r="CY15" s="9">
+        <f>COUNTIF(D15:CX15,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ15" s="9">
         <f>COUNTIF(D15:CX15,"בית")</f>
         <v/>
       </c>
-      <c r="CZ15" s="9">
-        <f>COUNTIF(D15:CX15,"בסיס")</f>
+      <c r="DA15" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D15:CX15="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB15" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D15:CX15="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2844,11 +3024,19 @@
       <c r="CW16" s="8" t="n"/>
       <c r="CX16" s="8" t="n"/>
       <c r="CY16" s="9">
+        <f>COUNTIF(D16:CX16,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ16" s="9">
         <f>COUNTIF(D16:CX16,"בית")</f>
         <v/>
       </c>
-      <c r="CZ16" s="9">
-        <f>COUNTIF(D16:CX16,"בסיס")</f>
+      <c r="DA16" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D16:CX16="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB16" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D16:CX16="בית"))</f>
         <v/>
       </c>
     </row>
@@ -2964,11 +3152,19 @@
       <c r="CW17" s="8" t="n"/>
       <c r="CX17" s="8" t="n"/>
       <c r="CY17" s="9">
+        <f>COUNTIF(D17:CX17,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ17" s="9">
         <f>COUNTIF(D17:CX17,"בית")</f>
         <v/>
       </c>
-      <c r="CZ17" s="9">
-        <f>COUNTIF(D17:CX17,"בסיס")</f>
+      <c r="DA17" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D17:CX17="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB17" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D17:CX17="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3080,11 +3276,19 @@
       <c r="CW18" s="8" t="n"/>
       <c r="CX18" s="8" t="n"/>
       <c r="CY18" s="9">
+        <f>COUNTIF(D18:CX18,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ18" s="9">
         <f>COUNTIF(D18:CX18,"בית")</f>
         <v/>
       </c>
-      <c r="CZ18" s="9">
-        <f>COUNTIF(D18:CX18,"בסיס")</f>
+      <c r="DA18" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D18:CX18="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB18" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D18:CX18="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3196,11 +3400,19 @@
       <c r="CW19" s="8" t="n"/>
       <c r="CX19" s="8" t="n"/>
       <c r="CY19" s="9">
+        <f>COUNTIF(D19:CX19,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ19" s="9">
         <f>COUNTIF(D19:CX19,"בית")</f>
         <v/>
       </c>
-      <c r="CZ19" s="9">
-        <f>COUNTIF(D19:CX19,"בסיס")</f>
+      <c r="DA19" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D19:CX19="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB19" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D19:CX19="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3316,11 +3528,19 @@
       <c r="CW20" s="8" t="n"/>
       <c r="CX20" s="8" t="n"/>
       <c r="CY20" s="9">
+        <f>COUNTIF(D20:CX20,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ20" s="9">
         <f>COUNTIF(D20:CX20,"בית")</f>
         <v/>
       </c>
-      <c r="CZ20" s="9">
-        <f>COUNTIF(D20:CX20,"בסיס")</f>
+      <c r="DA20" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D20:CX20="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB20" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D20:CX20="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3436,11 +3656,19 @@
       <c r="CW21" s="8" t="n"/>
       <c r="CX21" s="8" t="n"/>
       <c r="CY21" s="9">
+        <f>COUNTIF(D21:CX21,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ21" s="9">
         <f>COUNTIF(D21:CX21,"בית")</f>
         <v/>
       </c>
-      <c r="CZ21" s="9">
-        <f>COUNTIF(D21:CX21,"בסיס")</f>
+      <c r="DA21" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D21:CX21="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB21" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D21:CX21="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3556,11 +3784,19 @@
       <c r="CW22" s="8" t="n"/>
       <c r="CX22" s="8" t="n"/>
       <c r="CY22" s="9">
+        <f>COUNTIF(D22:CX22,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ22" s="9">
         <f>COUNTIF(D22:CX22,"בית")</f>
         <v/>
       </c>
-      <c r="CZ22" s="9">
-        <f>COUNTIF(D22:CX22,"בסיס")</f>
+      <c r="DA22" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D22:CX22="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB22" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D22:CX22="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3672,11 +3908,19 @@
       <c r="CW23" s="8" t="n"/>
       <c r="CX23" s="8" t="n"/>
       <c r="CY23" s="9">
+        <f>COUNTIF(D23:CX23,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ23" s="9">
         <f>COUNTIF(D23:CX23,"בית")</f>
         <v/>
       </c>
-      <c r="CZ23" s="9">
-        <f>COUNTIF(D23:CX23,"בסיס")</f>
+      <c r="DA23" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D23:CX23="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB23" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D23:CX23="בית"))</f>
         <v/>
       </c>
     </row>
@@ -3792,11 +4036,19 @@
       <c r="CW24" s="8" t="n"/>
       <c r="CX24" s="8" t="n"/>
       <c r="CY24" s="9">
+        <f>COUNTIF(D24:CX24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CZ24" s="9">
         <f>COUNTIF(D24:CX24,"בית")</f>
         <v/>
       </c>
-      <c r="CZ24" s="9">
-        <f>COUNTIF(D24:CX24,"בסיס")</f>
+      <c r="DA24" s="9">
+        <f>SUMPRODUCT($D$30:$CX$30,--(D24:CX24="בית"))</f>
+        <v/>
+      </c>
+      <c r="DB24" s="9">
+        <f>SUMPRODUCT($D$31:$CX$31,--(D24:CX24="בית"))</f>
         <v/>
       </c>
     </row>
@@ -4206,427 +4458,1919 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
+          <t>נשקייה בבסיס</t>
+        </is>
+      </c>
+      <c r="D26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",D4:D24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="E26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",E4:E24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="F26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",F4:F24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",G4:G24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="H26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",H4:H24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="I26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",I4:I24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="J26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",J4:J24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="K26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",K4:K24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="L26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",L4:L24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="M26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",M4:M24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="N26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",N4:N24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="O26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",O4:O24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="P26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",P4:P24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",Q4:Q24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="R26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",R4:R24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="S26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",S4:S24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="T26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",T4:T24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="U26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",U4:U24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="V26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",V4:V24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="W26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",W4:W24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="X26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",X4:X24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Y26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",Y4:Y24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Z26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",Z4:Z24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AA26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AA4:AA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AB26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AB4:AB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AC26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AC4:AC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AD26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AD4:AD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AE26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AE4:AE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AF26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AF4:AF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AG26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AG4:AG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AH26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AH4:AH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AI26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AI4:AI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AJ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AJ4:AJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AK26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AK4:AK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AL26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AL4:AL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AM26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AM4:AM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AN26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AN4:AN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AO26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AO4:AO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AP26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AP4:AP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AQ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AQ4:AQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AR26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AR4:AR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AS26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AS4:AS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AT26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AT4:AT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AU26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AU4:AU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AV26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AV4:AV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AW26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AW4:AW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AX26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AX4:AX24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AY26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AY4:AY24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AZ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",AZ4:AZ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BA26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BA4:BA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BB26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BB4:BB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BC26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BC4:BC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BD26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BD4:BD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BE26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BE4:BE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BF26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BF4:BF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BG26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BG4:BG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BH26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BH4:BH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BI26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BI4:BI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BJ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BJ4:BJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BK26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BK4:BK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BL26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BL4:BL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BM26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BM4:BM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BN26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BN4:BN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BO26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BO4:BO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BP26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BP4:BP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BQ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BQ4:BQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BR26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BR4:BR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BS26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BS4:BS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BT26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BT4:BT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BU26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BU4:BU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BV26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BV4:BV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BW26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BW4:BW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BX26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BX4:BX24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BY26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BY4:BY24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BZ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",BZ4:BZ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CA26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CA4:CA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CB26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CB4:CB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CC26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CC4:CC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CD26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CD4:CD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CE26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CE4:CE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CF26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CF4:CF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CG26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CG4:CG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CH26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CH4:CH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CI26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CI4:CI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CJ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CJ4:CJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CK26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CK4:CK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CL26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CL4:CL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CM26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CM4:CM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CN26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CN4:CN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CO26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CO4:CO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CP26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CP4:CP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CQ26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CQ4:CQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CR26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CR4:CR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CS26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CS4:CS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CT26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CT4:CT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CU26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CU4:CU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CV26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CV4:CV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CW26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CW4:CW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CX26" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*נשקייה*",CX4:CX24,"בסיס")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>אפסנאות בבסיס</t>
+        </is>
+      </c>
+      <c r="D27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",D4:D24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="E27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",E4:E24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="F27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",F4:F24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="G27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",G4:G24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="H27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",H4:H24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="I27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",I4:I24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="J27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",J4:J24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="K27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",K4:K24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="L27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",L4:L24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="M27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",M4:M24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="N27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",N4:N24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="O27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",O4:O24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="P27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",P4:P24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",Q4:Q24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="R27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",R4:R24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="S27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",S4:S24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="T27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",T4:T24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="U27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",U4:U24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="V27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",V4:V24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="W27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",W4:W24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="X27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",X4:X24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Y27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",Y4:Y24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="Z27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",Z4:Z24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AA27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AA4:AA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AB27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AB4:AB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AC27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AC4:AC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AD27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AD4:AD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AE27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AE4:AE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AF27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AF4:AF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AG27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AG4:AG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AH27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AH4:AH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AI27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AI4:AI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AJ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AJ4:AJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AK27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AK4:AK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AL27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AL4:AL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AM27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AM4:AM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AN27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AN4:AN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AO27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AO4:AO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AP27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AP4:AP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AQ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AQ4:AQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AR27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AR4:AR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AS27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AS4:AS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AT27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AT4:AT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AU27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AU4:AU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AV27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AV4:AV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AW27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AW4:AW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AX27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AX4:AX24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AY27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AY4:AY24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="AZ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",AZ4:AZ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BA27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BA4:BA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BB27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BB4:BB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BC27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BC4:BC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BD27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BD4:BD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BE27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BE4:BE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BF27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BF4:BF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BG27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BG4:BG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BH27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BH4:BH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BI27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BI4:BI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BJ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BJ4:BJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BK27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BK4:BK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BL27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BL4:BL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BM27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BM4:BM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BN27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BN4:BN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BO27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BO4:BO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BP27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BP4:BP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BQ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BQ4:BQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BR27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BR4:BR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BS27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BS4:BS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BT27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BT4:BT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BU27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BU4:BU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BV27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BV4:BV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BW27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BW4:BW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BX27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BX4:BX24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BY27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BY4:BY24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="BZ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",BZ4:BZ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CA27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CA4:CA24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CB27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CB4:CB24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CC27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CC4:CC24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CD27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CD4:CD24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CE27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CE4:CE24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CF27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CF4:CF24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CG27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CG4:CG24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CH27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CH4:CH24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CI27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CI4:CI24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CJ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CJ4:CJ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CK27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CK4:CK24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CL27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CL4:CL24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CM27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CM4:CM24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CN27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CN4:CN24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CO27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CO4:CO24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CP27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CP4:CP24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CQ27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CQ4:CQ24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CR27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CR4:CR24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CS27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CS4:CS24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CT27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CT4:CT24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CU27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CU4:CU24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CV27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CV4:CV24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CW27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CW4:CW24,"בסיס")</f>
+        <v/>
+      </c>
+      <c r="CX27" s="11">
+        <f>COUNTIFS($B$4:$B$24,"*אפסנאות*",CX4:CX24,"בסיס")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
           <t>סה"כ בבית</t>
         </is>
       </c>
-      <c r="D26" s="11">
+      <c r="D28" s="11">
         <f>COUNTIF(D4:D24,"בית")</f>
         <v/>
       </c>
-      <c r="E26" s="11">
+      <c r="E28" s="11">
         <f>COUNTIF(E4:E24,"בית")</f>
         <v/>
       </c>
-      <c r="F26" s="11">
+      <c r="F28" s="11">
         <f>COUNTIF(F4:F24,"בית")</f>
         <v/>
       </c>
-      <c r="G26" s="11">
+      <c r="G28" s="11">
         <f>COUNTIF(G4:G24,"בית")</f>
         <v/>
       </c>
-      <c r="H26" s="11">
+      <c r="H28" s="11">
         <f>COUNTIF(H4:H24,"בית")</f>
         <v/>
       </c>
-      <c r="I26" s="11">
+      <c r="I28" s="11">
         <f>COUNTIF(I4:I24,"בית")</f>
         <v/>
       </c>
-      <c r="J26" s="11">
+      <c r="J28" s="11">
         <f>COUNTIF(J4:J24,"בית")</f>
         <v/>
       </c>
-      <c r="K26" s="11">
+      <c r="K28" s="11">
         <f>COUNTIF(K4:K24,"בית")</f>
         <v/>
       </c>
-      <c r="L26" s="11">
+      <c r="L28" s="11">
         <f>COUNTIF(L4:L24,"בית")</f>
         <v/>
       </c>
-      <c r="M26" s="11">
+      <c r="M28" s="11">
         <f>COUNTIF(M4:M24,"בית")</f>
         <v/>
       </c>
-      <c r="N26" s="11">
+      <c r="N28" s="11">
         <f>COUNTIF(N4:N24,"בית")</f>
         <v/>
       </c>
-      <c r="O26" s="11">
+      <c r="O28" s="11">
         <f>COUNTIF(O4:O24,"בית")</f>
         <v/>
       </c>
-      <c r="P26" s="11">
+      <c r="P28" s="11">
         <f>COUNTIF(P4:P24,"בית")</f>
         <v/>
       </c>
-      <c r="Q26" s="11">
+      <c r="Q28" s="11">
         <f>COUNTIF(Q4:Q24,"בית")</f>
         <v/>
       </c>
-      <c r="R26" s="11">
+      <c r="R28" s="11">
         <f>COUNTIF(R4:R24,"בית")</f>
         <v/>
       </c>
-      <c r="S26" s="11">
+      <c r="S28" s="11">
         <f>COUNTIF(S4:S24,"בית")</f>
         <v/>
       </c>
-      <c r="T26" s="11">
+      <c r="T28" s="11">
         <f>COUNTIF(T4:T24,"בית")</f>
         <v/>
       </c>
-      <c r="U26" s="11">
+      <c r="U28" s="11">
         <f>COUNTIF(U4:U24,"בית")</f>
         <v/>
       </c>
-      <c r="V26" s="11">
+      <c r="V28" s="11">
         <f>COUNTIF(V4:V24,"בית")</f>
         <v/>
       </c>
-      <c r="W26" s="11">
+      <c r="W28" s="11">
         <f>COUNTIF(W4:W24,"בית")</f>
         <v/>
       </c>
-      <c r="X26" s="11">
+      <c r="X28" s="11">
         <f>COUNTIF(X4:X24,"בית")</f>
         <v/>
       </c>
-      <c r="Y26" s="11">
+      <c r="Y28" s="11">
         <f>COUNTIF(Y4:Y24,"בית")</f>
         <v/>
       </c>
-      <c r="Z26" s="11">
+      <c r="Z28" s="11">
         <f>COUNTIF(Z4:Z24,"בית")</f>
         <v/>
       </c>
-      <c r="AA26" s="11">
+      <c r="AA28" s="11">
         <f>COUNTIF(AA4:AA24,"בית")</f>
         <v/>
       </c>
-      <c r="AB26" s="11">
+      <c r="AB28" s="11">
         <f>COUNTIF(AB4:AB24,"בית")</f>
         <v/>
       </c>
-      <c r="AC26" s="11">
+      <c r="AC28" s="11">
         <f>COUNTIF(AC4:AC24,"בית")</f>
         <v/>
       </c>
-      <c r="AD26" s="11">
+      <c r="AD28" s="11">
         <f>COUNTIF(AD4:AD24,"בית")</f>
         <v/>
       </c>
-      <c r="AE26" s="11">
+      <c r="AE28" s="11">
         <f>COUNTIF(AE4:AE24,"בית")</f>
         <v/>
       </c>
-      <c r="AF26" s="11">
+      <c r="AF28" s="11">
         <f>COUNTIF(AF4:AF24,"בית")</f>
         <v/>
       </c>
-      <c r="AG26" s="11">
+      <c r="AG28" s="11">
         <f>COUNTIF(AG4:AG24,"בית")</f>
         <v/>
       </c>
-      <c r="AH26" s="11">
+      <c r="AH28" s="11">
         <f>COUNTIF(AH4:AH24,"בית")</f>
         <v/>
       </c>
-      <c r="AI26" s="11">
+      <c r="AI28" s="11">
         <f>COUNTIF(AI4:AI24,"בית")</f>
         <v/>
       </c>
-      <c r="AJ26" s="11">
+      <c r="AJ28" s="11">
         <f>COUNTIF(AJ4:AJ24,"בית")</f>
         <v/>
       </c>
-      <c r="AK26" s="11">
+      <c r="AK28" s="11">
         <f>COUNTIF(AK4:AK24,"בית")</f>
         <v/>
       </c>
-      <c r="AL26" s="11">
+      <c r="AL28" s="11">
         <f>COUNTIF(AL4:AL24,"בית")</f>
         <v/>
       </c>
-      <c r="AM26" s="11">
+      <c r="AM28" s="11">
         <f>COUNTIF(AM4:AM24,"בית")</f>
         <v/>
       </c>
-      <c r="AN26" s="11">
+      <c r="AN28" s="11">
         <f>COUNTIF(AN4:AN24,"בית")</f>
         <v/>
       </c>
-      <c r="AO26" s="11">
+      <c r="AO28" s="11">
         <f>COUNTIF(AO4:AO24,"בית")</f>
         <v/>
       </c>
-      <c r="AP26" s="11">
+      <c r="AP28" s="11">
         <f>COUNTIF(AP4:AP24,"בית")</f>
         <v/>
       </c>
-      <c r="AQ26" s="11">
+      <c r="AQ28" s="11">
         <f>COUNTIF(AQ4:AQ24,"בית")</f>
         <v/>
       </c>
-      <c r="AR26" s="11">
+      <c r="AR28" s="11">
         <f>COUNTIF(AR4:AR24,"בית")</f>
         <v/>
       </c>
-      <c r="AS26" s="11">
+      <c r="AS28" s="11">
         <f>COUNTIF(AS4:AS24,"בית")</f>
         <v/>
       </c>
-      <c r="AT26" s="11">
+      <c r="AT28" s="11">
         <f>COUNTIF(AT4:AT24,"בית")</f>
         <v/>
       </c>
-      <c r="AU26" s="11">
+      <c r="AU28" s="11">
         <f>COUNTIF(AU4:AU24,"בית")</f>
         <v/>
       </c>
-      <c r="AV26" s="11">
+      <c r="AV28" s="11">
         <f>COUNTIF(AV4:AV24,"בית")</f>
         <v/>
       </c>
-      <c r="AW26" s="11">
+      <c r="AW28" s="11">
         <f>COUNTIF(AW4:AW24,"בית")</f>
         <v/>
       </c>
-      <c r="AX26" s="11">
+      <c r="AX28" s="11">
         <f>COUNTIF(AX4:AX24,"בית")</f>
         <v/>
       </c>
-      <c r="AY26" s="11">
+      <c r="AY28" s="11">
         <f>COUNTIF(AY4:AY24,"בית")</f>
         <v/>
       </c>
-      <c r="AZ26" s="11">
+      <c r="AZ28" s="11">
         <f>COUNTIF(AZ4:AZ24,"בית")</f>
         <v/>
       </c>
-      <c r="BA26" s="11">
+      <c r="BA28" s="11">
         <f>COUNTIF(BA4:BA24,"בית")</f>
         <v/>
       </c>
-      <c r="BB26" s="11">
+      <c r="BB28" s="11">
         <f>COUNTIF(BB4:BB24,"בית")</f>
         <v/>
       </c>
-      <c r="BC26" s="11">
+      <c r="BC28" s="11">
         <f>COUNTIF(BC4:BC24,"בית")</f>
         <v/>
       </c>
-      <c r="BD26" s="11">
+      <c r="BD28" s="11">
         <f>COUNTIF(BD4:BD24,"בית")</f>
         <v/>
       </c>
-      <c r="BE26" s="11">
+      <c r="BE28" s="11">
         <f>COUNTIF(BE4:BE24,"בית")</f>
         <v/>
       </c>
-      <c r="BF26" s="11">
+      <c r="BF28" s="11">
         <f>COUNTIF(BF4:BF24,"בית")</f>
         <v/>
       </c>
-      <c r="BG26" s="11">
+      <c r="BG28" s="11">
         <f>COUNTIF(BG4:BG24,"בית")</f>
         <v/>
       </c>
-      <c r="BH26" s="11">
+      <c r="BH28" s="11">
         <f>COUNTIF(BH4:BH24,"בית")</f>
         <v/>
       </c>
-      <c r="BI26" s="11">
+      <c r="BI28" s="11">
         <f>COUNTIF(BI4:BI24,"בית")</f>
         <v/>
       </c>
-      <c r="BJ26" s="11">
+      <c r="BJ28" s="11">
         <f>COUNTIF(BJ4:BJ24,"בית")</f>
         <v/>
       </c>
-      <c r="BK26" s="11">
+      <c r="BK28" s="11">
         <f>COUNTIF(BK4:BK24,"בית")</f>
         <v/>
       </c>
-      <c r="BL26" s="11">
+      <c r="BL28" s="11">
         <f>COUNTIF(BL4:BL24,"בית")</f>
         <v/>
       </c>
-      <c r="BM26" s="11">
+      <c r="BM28" s="11">
         <f>COUNTIF(BM4:BM24,"בית")</f>
         <v/>
       </c>
-      <c r="BN26" s="11">
+      <c r="BN28" s="11">
         <f>COUNTIF(BN4:BN24,"בית")</f>
         <v/>
       </c>
-      <c r="BO26" s="11">
+      <c r="BO28" s="11">
         <f>COUNTIF(BO4:BO24,"בית")</f>
         <v/>
       </c>
-      <c r="BP26" s="11">
+      <c r="BP28" s="11">
         <f>COUNTIF(BP4:BP24,"בית")</f>
         <v/>
       </c>
-      <c r="BQ26" s="11">
+      <c r="BQ28" s="11">
         <f>COUNTIF(BQ4:BQ24,"בית")</f>
         <v/>
       </c>
-      <c r="BR26" s="11">
+      <c r="BR28" s="11">
         <f>COUNTIF(BR4:BR24,"בית")</f>
         <v/>
       </c>
-      <c r="BS26" s="11">
+      <c r="BS28" s="11">
         <f>COUNTIF(BS4:BS24,"בית")</f>
         <v/>
       </c>
-      <c r="BT26" s="11">
+      <c r="BT28" s="11">
         <f>COUNTIF(BT4:BT24,"בית")</f>
         <v/>
       </c>
-      <c r="BU26" s="11">
+      <c r="BU28" s="11">
         <f>COUNTIF(BU4:BU24,"בית")</f>
         <v/>
       </c>
-      <c r="BV26" s="11">
+      <c r="BV28" s="11">
         <f>COUNTIF(BV4:BV24,"בית")</f>
         <v/>
       </c>
-      <c r="BW26" s="11">
+      <c r="BW28" s="11">
         <f>COUNTIF(BW4:BW24,"בית")</f>
         <v/>
       </c>
-      <c r="BX26" s="11">
+      <c r="BX28" s="11">
         <f>COUNTIF(BX4:BX24,"בית")</f>
         <v/>
       </c>
-      <c r="BY26" s="11">
+      <c r="BY28" s="11">
         <f>COUNTIF(BY4:BY24,"בית")</f>
         <v/>
       </c>
-      <c r="BZ26" s="11">
+      <c r="BZ28" s="11">
         <f>COUNTIF(BZ4:BZ24,"בית")</f>
         <v/>
       </c>
-      <c r="CA26" s="11">
+      <c r="CA28" s="11">
         <f>COUNTIF(CA4:CA24,"בית")</f>
         <v/>
       </c>
-      <c r="CB26" s="11">
+      <c r="CB28" s="11">
         <f>COUNTIF(CB4:CB24,"בית")</f>
         <v/>
       </c>
-      <c r="CC26" s="11">
+      <c r="CC28" s="11">
         <f>COUNTIF(CC4:CC24,"בית")</f>
         <v/>
       </c>
-      <c r="CD26" s="11">
+      <c r="CD28" s="11">
         <f>COUNTIF(CD4:CD24,"בית")</f>
         <v/>
       </c>
-      <c r="CE26" s="11">
+      <c r="CE28" s="11">
         <f>COUNTIF(CE4:CE24,"בית")</f>
         <v/>
       </c>
-      <c r="CF26" s="11">
+      <c r="CF28" s="11">
         <f>COUNTIF(CF4:CF24,"בית")</f>
         <v/>
       </c>
-      <c r="CG26" s="11">
+      <c r="CG28" s="11">
         <f>COUNTIF(CG4:CG24,"בית")</f>
         <v/>
       </c>
-      <c r="CH26" s="11">
+      <c r="CH28" s="11">
         <f>COUNTIF(CH4:CH24,"בית")</f>
         <v/>
       </c>
-      <c r="CI26" s="11">
+      <c r="CI28" s="11">
         <f>COUNTIF(CI4:CI24,"בית")</f>
         <v/>
       </c>
-      <c r="CJ26" s="11">
+      <c r="CJ28" s="11">
         <f>COUNTIF(CJ4:CJ24,"בית")</f>
         <v/>
       </c>
-      <c r="CK26" s="11">
+      <c r="CK28" s="11">
         <f>COUNTIF(CK4:CK24,"בית")</f>
         <v/>
       </c>
-      <c r="CL26" s="11">
+      <c r="CL28" s="11">
         <f>COUNTIF(CL4:CL24,"בית")</f>
         <v/>
       </c>
-      <c r="CM26" s="11">
+      <c r="CM28" s="11">
         <f>COUNTIF(CM4:CM24,"בית")</f>
         <v/>
       </c>
-      <c r="CN26" s="11">
+      <c r="CN28" s="11">
         <f>COUNTIF(CN4:CN24,"בית")</f>
         <v/>
       </c>
-      <c r="CO26" s="11">
+      <c r="CO28" s="11">
         <f>COUNTIF(CO4:CO24,"בית")</f>
         <v/>
       </c>
-      <c r="CP26" s="11">
+      <c r="CP28" s="11">
         <f>COUNTIF(CP4:CP24,"בית")</f>
         <v/>
       </c>
-      <c r="CQ26" s="11">
+      <c r="CQ28" s="11">
         <f>COUNTIF(CQ4:CQ24,"בית")</f>
         <v/>
       </c>
-      <c r="CR26" s="11">
+      <c r="CR28" s="11">
         <f>COUNTIF(CR4:CR24,"בית")</f>
         <v/>
       </c>
-      <c r="CS26" s="11">
+      <c r="CS28" s="11">
         <f>COUNTIF(CS4:CS24,"בית")</f>
         <v/>
       </c>
-      <c r="CT26" s="11">
+      <c r="CT28" s="11">
         <f>COUNTIF(CT4:CT24,"בית")</f>
         <v/>
       </c>
-      <c r="CU26" s="11">
+      <c r="CU28" s="11">
         <f>COUNTIF(CU4:CU24,"בית")</f>
         <v/>
       </c>
-      <c r="CV26" s="11">
+      <c r="CV28" s="11">
         <f>COUNTIF(CV4:CV24,"בית")</f>
         <v/>
       </c>
-      <c r="CW26" s="11">
+      <c r="CW28" s="11">
         <f>COUNTIF(CW4:CW24,"בית")</f>
         <v/>
       </c>
-      <c r="CX26" s="11">
+      <c r="CX28" s="11">
         <f>COUNTIF(CX4:CX24,"בית")</f>
         <v/>
+      </c>
+    </row>
+    <row r="30" hidden="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[דגל שבת]</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>1</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF30" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM30" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT30" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" hidden="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[דגל חג]</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CT31" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>הגדרות מצבה (ניתן לעריכה):</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>מינימום בבסיס</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>מינימום נשקייה</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>מינימום אפסנאות</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="BU2:CX2"/>
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A1:DB1"/>
     <mergeCell ref="K2:AO2"/>
     <mergeCell ref="AP2:BT2"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="D2:J2"/>
     <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A1:CZ1"/>
   </mergeCells>
+  <conditionalFormatting sqref="D25:CX25">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>$B$33</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D26:CX26">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
+      <formula>$B$34</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D27:CX27">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
+      <formula>$B$35</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D4:CX24">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"בסיס"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
       <formula>"בית"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"בסיס"</formula>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="3">
+      <formula>"חופשה"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4">
+      <formula>"גימלים"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="5">
+      <formula>"קורס"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
+      <formula>"ת״ש"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="DA4:DA24">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00C6EFCE"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00FFC7CE"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="D4:CX24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"בית,בסיס"</formula1>
+      <formula1>"בסיס,בית,חופשה,גימלים,קורס,ת״ש"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4639,57 +6383,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>מקרא - שבצק יציאות</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="n"/>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>שבת / ערב שבת</t>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>כותרת תאריך:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="n"/>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>חג</t>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>שבת / ערב שבת</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>יום בית</t>
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>חג</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n"/>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>יום בסיס</t>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>סטטוס תא:</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="n"/>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>יום רגיל (נייטרלי)</t>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>בסיס</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>חופשה</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>גימלים</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n"/>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>קורס</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>ת״ש</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>התראות:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="n"/>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>מתחת לסף מצבה (אדום אוטומטי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>ספי המצבה נקבעים בגיליון השבצק בבלוק "הגדרות מצבה".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add personal-conversation tracking sheet
A short per-soldier log: talked yes/no (color-coded), date, topic, notes,
with running totals of completed and pending conversations.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/shavtzak_yetziot.xlsx
+++ b/shavtzak_yetziot.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="שבצק יציאות" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="מקרא" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="שיחות עם חיילים" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -185,6 +186,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6500,4 +6504,427 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>שיחות אישיות עם חיילים</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>שם</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>תפקיד</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>שוחחת?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>תאריך שיחה</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>נושא</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>הערות</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>איתי עוזיאל</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>קלג</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="9" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>אורי עוזיאל</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>סמל נשקייה</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>ינון איזון</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>שי ארנלדס</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>איתי שמש</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>אביעד כהן</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>אזוגי נתנאל</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>ניב סורוקר</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>צבי לונדין</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>יוסף חגואל</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>אדם ממן</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>סמל אפסנאות</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>גבריאל יעקוביאן</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>יקיר אלימלך</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>יוסי כהן</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה-רחפנים</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>רון בן שושן</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>דוד שמחי</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>לב גינזבורג</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>נשקייה</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>יעקב גרמאי</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>עידן אשטון</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>עומר נוימן</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>דוד עבאדה</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>אפסנאות</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>סה"כ שוחחו:</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>COUNTIF(C3:C23,"כן")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>נותרו לשיחה:</t>
+        </is>
+      </c>
+      <c r="B26" s="25">
+        <f>COUNTIF(C3:C23,"לא")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C3:C23">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"כן"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"לא"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="C3:C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"כן,לא"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Force FF alpha on conditional-formatting fills and pre-fill demo statuses
Some viewers (Google Sheets, some mobile previews) drop fills with
implicit 00 alpha. Explicit FF alpha keeps the status colors visible
everywhere. Also pre-fill six demo cells so the user immediately sees
the per-status coloring working when opening the workbook.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/shavtzak_yetziot.xlsx
+++ b/shavtzak_yetziot.xlsx
@@ -193,7 +193,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <font>
         <b val="1"/>
@@ -201,14 +201,49 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FF5050"/>
+          <fgColor rgb="FFFF5050"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00BDD7EE"/>
+          <fgColor rgb="FFBDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA9D08E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB4A7D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -222,28 +257,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00A9D08E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00B4A7D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1392,14 +1406,42 @@
         </is>
       </c>
       <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>בסיס</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>בית</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>חופשה</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>גימלים</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>קורס</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>ת״ש</t>
+        </is>
+      </c>
       <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>← דוגמה למחיקה</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n"/>
@@ -6986,9 +7028,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="00C6EFCE"/>
-        <color rgb="00FFEB9C"/>
-        <color rgb="00FFC7CE"/>
+        <color rgb="FFC6EFCE"/>
+        <color rgb="FFFFEB9C"/>
+        <color rgb="FFFFC7CE"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -7593,10 +7635,10 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C28">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="7">
       <formula>"כן"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="8">
       <formula>"לא"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Add direct fills to demo row and set both fg/bg on CF dxf
The auto-coloring still depends on the viewer supporting conditional
formatting. To guarantee the user sees the six status colors when they
open the file (including preview-only viewers), paint the demo row
directly. Also set both fgColor and bgColor on the CF dxf for broader
viewer compatibility.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/shavtzak_yetziot.xlsx
+++ b/shavtzak_yetziot.xlsx
@@ -49,7 +49,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4A7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +192,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -179,13 +227,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -209,6 +257,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFBDD7EE"/>
+          <bgColor rgb="FFBDD7EE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -216,6 +265,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -223,6 +273,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFA9D08E"/>
+          <bgColor rgb="FFA9D08E"/>
         </patternFill>
       </fill>
     </dxf>
@@ -230,6 +281,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -237,6 +289,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFB4A7D6"/>
+          <bgColor rgb="FFB4A7D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -244,6 +297,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1411,33 +1465,33 @@
           <t>בסיס</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>בית</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>חופשה</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>גימלים</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>קורס</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>ת״ש</t>
         </is>
       </c>
       <c r="J4" s="8" t="n"/>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="15" t="inlineStr">
         <is>
           <t>← דוגמה למחיקה</t>
         </is>
@@ -1533,19 +1587,19 @@
       <c r="CV4" s="8" t="n"/>
       <c r="CW4" s="8" t="n"/>
       <c r="CX4" s="8" t="n"/>
-      <c r="CY4" s="9">
+      <c r="CY4" s="15">
         <f>COUNTIF(D4:CX4,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ4" s="9">
+      <c r="CZ4" s="15">
         <f>COUNTIF(D4:CX4,"בית")</f>
         <v/>
       </c>
-      <c r="DA4" s="9">
+      <c r="DA4" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D4:CX4="בית"))</f>
         <v/>
       </c>
-      <c r="DB4" s="9">
+      <c r="DB4" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D4:CX4="בית"))</f>
         <v/>
       </c>
@@ -1661,19 +1715,19 @@
       <c r="CV5" s="8" t="n"/>
       <c r="CW5" s="8" t="n"/>
       <c r="CX5" s="8" t="n"/>
-      <c r="CY5" s="9">
+      <c r="CY5" s="15">
         <f>COUNTIF(D5:CX5,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ5" s="9">
+      <c r="CZ5" s="15">
         <f>COUNTIF(D5:CX5,"בית")</f>
         <v/>
       </c>
-      <c r="DA5" s="9">
+      <c r="DA5" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D5:CX5="בית"))</f>
         <v/>
       </c>
-      <c r="DB5" s="9">
+      <c r="DB5" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D5:CX5="בית"))</f>
         <v/>
       </c>
@@ -1789,19 +1843,19 @@
       <c r="CV6" s="8" t="n"/>
       <c r="CW6" s="8" t="n"/>
       <c r="CX6" s="8" t="n"/>
-      <c r="CY6" s="9">
+      <c r="CY6" s="15">
         <f>COUNTIF(D6:CX6,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ6" s="9">
+      <c r="CZ6" s="15">
         <f>COUNTIF(D6:CX6,"בית")</f>
         <v/>
       </c>
-      <c r="DA6" s="9">
+      <c r="DA6" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D6:CX6="בית"))</f>
         <v/>
       </c>
-      <c r="DB6" s="9">
+      <c r="DB6" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D6:CX6="בית"))</f>
         <v/>
       </c>
@@ -1917,19 +1971,19 @@
       <c r="CV7" s="8" t="n"/>
       <c r="CW7" s="8" t="n"/>
       <c r="CX7" s="8" t="n"/>
-      <c r="CY7" s="9">
+      <c r="CY7" s="15">
         <f>COUNTIF(D7:CX7,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ7" s="9">
+      <c r="CZ7" s="15">
         <f>COUNTIF(D7:CX7,"בית")</f>
         <v/>
       </c>
-      <c r="DA7" s="9">
+      <c r="DA7" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D7:CX7="בית"))</f>
         <v/>
       </c>
-      <c r="DB7" s="9">
+      <c r="DB7" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D7:CX7="בית"))</f>
         <v/>
       </c>
@@ -2045,19 +2099,19 @@
       <c r="CV8" s="8" t="n"/>
       <c r="CW8" s="8" t="n"/>
       <c r="CX8" s="8" t="n"/>
-      <c r="CY8" s="9">
+      <c r="CY8" s="15">
         <f>COUNTIF(D8:CX8,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ8" s="9">
+      <c r="CZ8" s="15">
         <f>COUNTIF(D8:CX8,"בית")</f>
         <v/>
       </c>
-      <c r="DA8" s="9">
+      <c r="DA8" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D8:CX8="בית"))</f>
         <v/>
       </c>
-      <c r="DB8" s="9">
+      <c r="DB8" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D8:CX8="בית"))</f>
         <v/>
       </c>
@@ -2173,19 +2227,19 @@
       <c r="CV9" s="8" t="n"/>
       <c r="CW9" s="8" t="n"/>
       <c r="CX9" s="8" t="n"/>
-      <c r="CY9" s="9">
+      <c r="CY9" s="15">
         <f>COUNTIF(D9:CX9,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ9" s="9">
+      <c r="CZ9" s="15">
         <f>COUNTIF(D9:CX9,"בית")</f>
         <v/>
       </c>
-      <c r="DA9" s="9">
+      <c r="DA9" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D9:CX9="בית"))</f>
         <v/>
       </c>
-      <c r="DB9" s="9">
+      <c r="DB9" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D9:CX9="בית"))</f>
         <v/>
       </c>
@@ -2301,19 +2355,19 @@
       <c r="CV10" s="8" t="n"/>
       <c r="CW10" s="8" t="n"/>
       <c r="CX10" s="8" t="n"/>
-      <c r="CY10" s="9">
+      <c r="CY10" s="15">
         <f>COUNTIF(D10:CX10,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ10" s="9">
+      <c r="CZ10" s="15">
         <f>COUNTIF(D10:CX10,"בית")</f>
         <v/>
       </c>
-      <c r="DA10" s="9">
+      <c r="DA10" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D10:CX10="בית"))</f>
         <v/>
       </c>
-      <c r="DB10" s="9">
+      <c r="DB10" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D10:CX10="בית"))</f>
         <v/>
       </c>
@@ -2429,19 +2483,19 @@
       <c r="CV11" s="8" t="n"/>
       <c r="CW11" s="8" t="n"/>
       <c r="CX11" s="8" t="n"/>
-      <c r="CY11" s="9">
+      <c r="CY11" s="15">
         <f>COUNTIF(D11:CX11,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ11" s="9">
+      <c r="CZ11" s="15">
         <f>COUNTIF(D11:CX11,"בית")</f>
         <v/>
       </c>
-      <c r="DA11" s="9">
+      <c r="DA11" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D11:CX11="בית"))</f>
         <v/>
       </c>
-      <c r="DB11" s="9">
+      <c r="DB11" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D11:CX11="בית"))</f>
         <v/>
       </c>
@@ -2557,19 +2611,19 @@
       <c r="CV12" s="8" t="n"/>
       <c r="CW12" s="8" t="n"/>
       <c r="CX12" s="8" t="n"/>
-      <c r="CY12" s="9">
+      <c r="CY12" s="15">
         <f>COUNTIF(D12:CX12,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ12" s="9">
+      <c r="CZ12" s="15">
         <f>COUNTIF(D12:CX12,"בית")</f>
         <v/>
       </c>
-      <c r="DA12" s="9">
+      <c r="DA12" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D12:CX12="בית"))</f>
         <v/>
       </c>
-      <c r="DB12" s="9">
+      <c r="DB12" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D12:CX12="בית"))</f>
         <v/>
       </c>
@@ -2685,19 +2739,19 @@
       <c r="CV13" s="8" t="n"/>
       <c r="CW13" s="8" t="n"/>
       <c r="CX13" s="8" t="n"/>
-      <c r="CY13" s="9">
+      <c r="CY13" s="15">
         <f>COUNTIF(D13:CX13,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ13" s="9">
+      <c r="CZ13" s="15">
         <f>COUNTIF(D13:CX13,"בית")</f>
         <v/>
       </c>
-      <c r="DA13" s="9">
+      <c r="DA13" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D13:CX13="בית"))</f>
         <v/>
       </c>
-      <c r="DB13" s="9">
+      <c r="DB13" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D13:CX13="בית"))</f>
         <v/>
       </c>
@@ -2813,19 +2867,19 @@
       <c r="CV14" s="8" t="n"/>
       <c r="CW14" s="8" t="n"/>
       <c r="CX14" s="8" t="n"/>
-      <c r="CY14" s="9">
+      <c r="CY14" s="15">
         <f>COUNTIF(D14:CX14,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ14" s="9">
+      <c r="CZ14" s="15">
         <f>COUNTIF(D14:CX14,"בית")</f>
         <v/>
       </c>
-      <c r="DA14" s="9">
+      <c r="DA14" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D14:CX14="בית"))</f>
         <v/>
       </c>
-      <c r="DB14" s="9">
+      <c r="DB14" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D14:CX14="בית"))</f>
         <v/>
       </c>
@@ -2941,19 +2995,19 @@
       <c r="CV15" s="8" t="n"/>
       <c r="CW15" s="8" t="n"/>
       <c r="CX15" s="8" t="n"/>
-      <c r="CY15" s="9">
+      <c r="CY15" s="15">
         <f>COUNTIF(D15:CX15,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ15" s="9">
+      <c r="CZ15" s="15">
         <f>COUNTIF(D15:CX15,"בית")</f>
         <v/>
       </c>
-      <c r="DA15" s="9">
+      <c r="DA15" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D15:CX15="בית"))</f>
         <v/>
       </c>
-      <c r="DB15" s="9">
+      <c r="DB15" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D15:CX15="בית"))</f>
         <v/>
       </c>
@@ -3069,19 +3123,19 @@
       <c r="CV16" s="8" t="n"/>
       <c r="CW16" s="8" t="n"/>
       <c r="CX16" s="8" t="n"/>
-      <c r="CY16" s="9">
+      <c r="CY16" s="15">
         <f>COUNTIF(D16:CX16,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ16" s="9">
+      <c r="CZ16" s="15">
         <f>COUNTIF(D16:CX16,"בית")</f>
         <v/>
       </c>
-      <c r="DA16" s="9">
+      <c r="DA16" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D16:CX16="בית"))</f>
         <v/>
       </c>
-      <c r="DB16" s="9">
+      <c r="DB16" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D16:CX16="בית"))</f>
         <v/>
       </c>
@@ -3197,19 +3251,19 @@
       <c r="CV17" s="8" t="n"/>
       <c r="CW17" s="8" t="n"/>
       <c r="CX17" s="8" t="n"/>
-      <c r="CY17" s="9">
+      <c r="CY17" s="15">
         <f>COUNTIF(D17:CX17,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ17" s="9">
+      <c r="CZ17" s="15">
         <f>COUNTIF(D17:CX17,"בית")</f>
         <v/>
       </c>
-      <c r="DA17" s="9">
+      <c r="DA17" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D17:CX17="בית"))</f>
         <v/>
       </c>
-      <c r="DB17" s="9">
+      <c r="DB17" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D17:CX17="בית"))</f>
         <v/>
       </c>
@@ -3321,19 +3375,19 @@
       <c r="CV18" s="8" t="n"/>
       <c r="CW18" s="8" t="n"/>
       <c r="CX18" s="8" t="n"/>
-      <c r="CY18" s="9">
+      <c r="CY18" s="15">
         <f>COUNTIF(D18:CX18,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ18" s="9">
+      <c r="CZ18" s="15">
         <f>COUNTIF(D18:CX18,"בית")</f>
         <v/>
       </c>
-      <c r="DA18" s="9">
+      <c r="DA18" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D18:CX18="בית"))</f>
         <v/>
       </c>
-      <c r="DB18" s="9">
+      <c r="DB18" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D18:CX18="בית"))</f>
         <v/>
       </c>
@@ -3445,19 +3499,19 @@
       <c r="CV19" s="8" t="n"/>
       <c r="CW19" s="8" t="n"/>
       <c r="CX19" s="8" t="n"/>
-      <c r="CY19" s="9">
+      <c r="CY19" s="15">
         <f>COUNTIF(D19:CX19,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ19" s="9">
+      <c r="CZ19" s="15">
         <f>COUNTIF(D19:CX19,"בית")</f>
         <v/>
       </c>
-      <c r="DA19" s="9">
+      <c r="DA19" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D19:CX19="בית"))</f>
         <v/>
       </c>
-      <c r="DB19" s="9">
+      <c r="DB19" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D19:CX19="בית"))</f>
         <v/>
       </c>
@@ -3573,19 +3627,19 @@
       <c r="CV20" s="8" t="n"/>
       <c r="CW20" s="8" t="n"/>
       <c r="CX20" s="8" t="n"/>
-      <c r="CY20" s="9">
+      <c r="CY20" s="15">
         <f>COUNTIF(D20:CX20,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ20" s="9">
+      <c r="CZ20" s="15">
         <f>COUNTIF(D20:CX20,"בית")</f>
         <v/>
       </c>
-      <c r="DA20" s="9">
+      <c r="DA20" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D20:CX20="בית"))</f>
         <v/>
       </c>
-      <c r="DB20" s="9">
+      <c r="DB20" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D20:CX20="בית"))</f>
         <v/>
       </c>
@@ -3701,19 +3755,19 @@
       <c r="CV21" s="8" t="n"/>
       <c r="CW21" s="8" t="n"/>
       <c r="CX21" s="8" t="n"/>
-      <c r="CY21" s="9">
+      <c r="CY21" s="15">
         <f>COUNTIF(D21:CX21,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ21" s="9">
+      <c r="CZ21" s="15">
         <f>COUNTIF(D21:CX21,"בית")</f>
         <v/>
       </c>
-      <c r="DA21" s="9">
+      <c r="DA21" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D21:CX21="בית"))</f>
         <v/>
       </c>
-      <c r="DB21" s="9">
+      <c r="DB21" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D21:CX21="בית"))</f>
         <v/>
       </c>
@@ -3829,19 +3883,19 @@
       <c r="CV22" s="8" t="n"/>
       <c r="CW22" s="8" t="n"/>
       <c r="CX22" s="8" t="n"/>
-      <c r="CY22" s="9">
+      <c r="CY22" s="15">
         <f>COUNTIF(D22:CX22,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ22" s="9">
+      <c r="CZ22" s="15">
         <f>COUNTIF(D22:CX22,"בית")</f>
         <v/>
       </c>
-      <c r="DA22" s="9">
+      <c r="DA22" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D22:CX22="בית"))</f>
         <v/>
       </c>
-      <c r="DB22" s="9">
+      <c r="DB22" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D22:CX22="בית"))</f>
         <v/>
       </c>
@@ -3953,19 +4007,19 @@
       <c r="CV23" s="8" t="n"/>
       <c r="CW23" s="8" t="n"/>
       <c r="CX23" s="8" t="n"/>
-      <c r="CY23" s="9">
+      <c r="CY23" s="15">
         <f>COUNTIF(D23:CX23,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ23" s="9">
+      <c r="CZ23" s="15">
         <f>COUNTIF(D23:CX23,"בית")</f>
         <v/>
       </c>
-      <c r="DA23" s="9">
+      <c r="DA23" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D23:CX23="בית"))</f>
         <v/>
       </c>
-      <c r="DB23" s="9">
+      <c r="DB23" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D23:CX23="בית"))</f>
         <v/>
       </c>
@@ -4081,19 +4135,19 @@
       <c r="CV24" s="8" t="n"/>
       <c r="CW24" s="8" t="n"/>
       <c r="CX24" s="8" t="n"/>
-      <c r="CY24" s="9">
+      <c r="CY24" s="15">
         <f>COUNTIF(D24:CX24,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ24" s="9">
+      <c r="CZ24" s="15">
         <f>COUNTIF(D24:CX24,"בית")</f>
         <v/>
       </c>
-      <c r="DA24" s="9">
+      <c r="DA24" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D24:CX24="בית"))</f>
         <v/>
       </c>
-      <c r="DB24" s="9">
+      <c r="DB24" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D24:CX24="בית"))</f>
         <v/>
       </c>
@@ -4205,19 +4259,19 @@
       <c r="CV25" s="8" t="n"/>
       <c r="CW25" s="8" t="n"/>
       <c r="CX25" s="8" t="n"/>
-      <c r="CY25" s="9">
+      <c r="CY25" s="15">
         <f>COUNTIF(D25:CX25,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ25" s="9">
+      <c r="CZ25" s="15">
         <f>COUNTIF(D25:CX25,"בית")</f>
         <v/>
       </c>
-      <c r="DA25" s="9">
+      <c r="DA25" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D25:CX25="בית"))</f>
         <v/>
       </c>
-      <c r="DB25" s="9">
+      <c r="DB25" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D25:CX25="בית"))</f>
         <v/>
       </c>
@@ -4329,19 +4383,19 @@
       <c r="CV26" s="8" t="n"/>
       <c r="CW26" s="8" t="n"/>
       <c r="CX26" s="8" t="n"/>
-      <c r="CY26" s="9">
+      <c r="CY26" s="15">
         <f>COUNTIF(D26:CX26,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ26" s="9">
+      <c r="CZ26" s="15">
         <f>COUNTIF(D26:CX26,"בית")</f>
         <v/>
       </c>
-      <c r="DA26" s="9">
+      <c r="DA26" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D26:CX26="בית"))</f>
         <v/>
       </c>
-      <c r="DB26" s="9">
+      <c r="DB26" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D26:CX26="בית"))</f>
         <v/>
       </c>
@@ -4453,19 +4507,19 @@
       <c r="CV27" s="8" t="n"/>
       <c r="CW27" s="8" t="n"/>
       <c r="CX27" s="8" t="n"/>
-      <c r="CY27" s="9">
+      <c r="CY27" s="15">
         <f>COUNTIF(D27:CX27,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ27" s="9">
+      <c r="CZ27" s="15">
         <f>COUNTIF(D27:CX27,"בית")</f>
         <v/>
       </c>
-      <c r="DA27" s="9">
+      <c r="DA27" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D27:CX27="בית"))</f>
         <v/>
       </c>
-      <c r="DB27" s="9">
+      <c r="DB27" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D27:CX27="בית"))</f>
         <v/>
       </c>
@@ -4577,19 +4631,19 @@
       <c r="CV28" s="8" t="n"/>
       <c r="CW28" s="8" t="n"/>
       <c r="CX28" s="8" t="n"/>
-      <c r="CY28" s="9">
+      <c r="CY28" s="15">
         <f>COUNTIF(D28:CX28,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ28" s="9">
+      <c r="CZ28" s="15">
         <f>COUNTIF(D28:CX28,"בית")</f>
         <v/>
       </c>
-      <c r="DA28" s="9">
+      <c r="DA28" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D28:CX28="בית"))</f>
         <v/>
       </c>
-      <c r="DB28" s="9">
+      <c r="DB28" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D28:CX28="בית"))</f>
         <v/>
       </c>
@@ -4701,1631 +4755,1631 @@
       <c r="CV29" s="8" t="n"/>
       <c r="CW29" s="8" t="n"/>
       <c r="CX29" s="8" t="n"/>
-      <c r="CY29" s="9">
+      <c r="CY29" s="15">
         <f>COUNTIF(D29:CX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CZ29" s="9">
+      <c r="CZ29" s="15">
         <f>COUNTIF(D29:CX29,"בית")</f>
         <v/>
       </c>
-      <c r="DA29" s="9">
+      <c r="DA29" s="15">
         <f>SUMPRODUCT($D$35:$CX$35,--(D29:CX29="בית"))</f>
         <v/>
       </c>
-      <c r="DB29" s="9">
+      <c r="DB29" s="15">
         <f>SUMPRODUCT($D$36:$CX$36,--(D29:CX29="בית"))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>סה"כ בבסיס</t>
         </is>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="17">
         <f>COUNTIF(D4:D29,"בסיס")</f>
         <v/>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="17">
         <f>COUNTIF(E4:E29,"בסיס")</f>
         <v/>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="17">
         <f>COUNTIF(F4:F29,"בסיס")</f>
         <v/>
       </c>
-      <c r="G30" s="11">
+      <c r="G30" s="17">
         <f>COUNTIF(G4:G29,"בסיס")</f>
         <v/>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="17">
         <f>COUNTIF(H4:H29,"בסיס")</f>
         <v/>
       </c>
-      <c r="I30" s="11">
+      <c r="I30" s="17">
         <f>COUNTIF(I4:I29,"בסיס")</f>
         <v/>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="17">
         <f>COUNTIF(J4:J29,"בסיס")</f>
         <v/>
       </c>
-      <c r="K30" s="11">
+      <c r="K30" s="17">
         <f>COUNTIF(K4:K29,"בסיס")</f>
         <v/>
       </c>
-      <c r="L30" s="11">
+      <c r="L30" s="17">
         <f>COUNTIF(L4:L29,"בסיס")</f>
         <v/>
       </c>
-      <c r="M30" s="11">
+      <c r="M30" s="17">
         <f>COUNTIF(M4:M29,"בסיס")</f>
         <v/>
       </c>
-      <c r="N30" s="11">
+      <c r="N30" s="17">
         <f>COUNTIF(N4:N29,"בסיס")</f>
         <v/>
       </c>
-      <c r="O30" s="11">
+      <c r="O30" s="17">
         <f>COUNTIF(O4:O29,"בסיס")</f>
         <v/>
       </c>
-      <c r="P30" s="11">
+      <c r="P30" s="17">
         <f>COUNTIF(P4:P29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Q30" s="11">
+      <c r="Q30" s="17">
         <f>COUNTIF(Q4:Q29,"בסיס")</f>
         <v/>
       </c>
-      <c r="R30" s="11">
+      <c r="R30" s="17">
         <f>COUNTIF(R4:R29,"בסיס")</f>
         <v/>
       </c>
-      <c r="S30" s="11">
+      <c r="S30" s="17">
         <f>COUNTIF(S4:S29,"בסיס")</f>
         <v/>
       </c>
-      <c r="T30" s="11">
+      <c r="T30" s="17">
         <f>COUNTIF(T4:T29,"בסיס")</f>
         <v/>
       </c>
-      <c r="U30" s="11">
+      <c r="U30" s="17">
         <f>COUNTIF(U4:U29,"בסיס")</f>
         <v/>
       </c>
-      <c r="V30" s="11">
+      <c r="V30" s="17">
         <f>COUNTIF(V4:V29,"בסיס")</f>
         <v/>
       </c>
-      <c r="W30" s="11">
+      <c r="W30" s="17">
         <f>COUNTIF(W4:W29,"בסיס")</f>
         <v/>
       </c>
-      <c r="X30" s="11">
+      <c r="X30" s="17">
         <f>COUNTIF(X4:X29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Y30" s="11">
+      <c r="Y30" s="17">
         <f>COUNTIF(Y4:Y29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Z30" s="11">
+      <c r="Z30" s="17">
         <f>COUNTIF(Z4:Z29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AA30" s="11">
+      <c r="AA30" s="17">
         <f>COUNTIF(AA4:AA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AB30" s="11">
+      <c r="AB30" s="17">
         <f>COUNTIF(AB4:AB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AC30" s="11">
+      <c r="AC30" s="17">
         <f>COUNTIF(AC4:AC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AD30" s="11">
+      <c r="AD30" s="17">
         <f>COUNTIF(AD4:AD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AE30" s="11">
+      <c r="AE30" s="17">
         <f>COUNTIF(AE4:AE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AF30" s="11">
+      <c r="AF30" s="17">
         <f>COUNTIF(AF4:AF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AG30" s="11">
+      <c r="AG30" s="17">
         <f>COUNTIF(AG4:AG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AH30" s="11">
+      <c r="AH30" s="17">
         <f>COUNTIF(AH4:AH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AI30" s="11">
+      <c r="AI30" s="17">
         <f>COUNTIF(AI4:AI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AJ30" s="11">
+      <c r="AJ30" s="17">
         <f>COUNTIF(AJ4:AJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AK30" s="11">
+      <c r="AK30" s="17">
         <f>COUNTIF(AK4:AK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AL30" s="11">
+      <c r="AL30" s="17">
         <f>COUNTIF(AL4:AL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AM30" s="11">
+      <c r="AM30" s="17">
         <f>COUNTIF(AM4:AM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AN30" s="11">
+      <c r="AN30" s="17">
         <f>COUNTIF(AN4:AN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AO30" s="11">
+      <c r="AO30" s="17">
         <f>COUNTIF(AO4:AO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AP30" s="11">
+      <c r="AP30" s="17">
         <f>COUNTIF(AP4:AP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AQ30" s="11">
+      <c r="AQ30" s="17">
         <f>COUNTIF(AQ4:AQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AR30" s="11">
+      <c r="AR30" s="17">
         <f>COUNTIF(AR4:AR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AS30" s="11">
+      <c r="AS30" s="17">
         <f>COUNTIF(AS4:AS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AT30" s="11">
+      <c r="AT30" s="17">
         <f>COUNTIF(AT4:AT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AU30" s="11">
+      <c r="AU30" s="17">
         <f>COUNTIF(AU4:AU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AV30" s="11">
+      <c r="AV30" s="17">
         <f>COUNTIF(AV4:AV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AW30" s="11">
+      <c r="AW30" s="17">
         <f>COUNTIF(AW4:AW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AX30" s="11">
+      <c r="AX30" s="17">
         <f>COUNTIF(AX4:AX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AY30" s="11">
+      <c r="AY30" s="17">
         <f>COUNTIF(AY4:AY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AZ30" s="11">
+      <c r="AZ30" s="17">
         <f>COUNTIF(AZ4:AZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BA30" s="11">
+      <c r="BA30" s="17">
         <f>COUNTIF(BA4:BA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BB30" s="11">
+      <c r="BB30" s="17">
         <f>COUNTIF(BB4:BB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BC30" s="11">
+      <c r="BC30" s="17">
         <f>COUNTIF(BC4:BC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BD30" s="11">
+      <c r="BD30" s="17">
         <f>COUNTIF(BD4:BD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BE30" s="11">
+      <c r="BE30" s="17">
         <f>COUNTIF(BE4:BE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BF30" s="11">
+      <c r="BF30" s="17">
         <f>COUNTIF(BF4:BF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BG30" s="11">
+      <c r="BG30" s="17">
         <f>COUNTIF(BG4:BG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BH30" s="11">
+      <c r="BH30" s="17">
         <f>COUNTIF(BH4:BH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BI30" s="11">
+      <c r="BI30" s="17">
         <f>COUNTIF(BI4:BI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BJ30" s="11">
+      <c r="BJ30" s="17">
         <f>COUNTIF(BJ4:BJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BK30" s="11">
+      <c r="BK30" s="17">
         <f>COUNTIF(BK4:BK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BL30" s="11">
+      <c r="BL30" s="17">
         <f>COUNTIF(BL4:BL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BM30" s="11">
+      <c r="BM30" s="17">
         <f>COUNTIF(BM4:BM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BN30" s="11">
+      <c r="BN30" s="17">
         <f>COUNTIF(BN4:BN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BO30" s="11">
+      <c r="BO30" s="17">
         <f>COUNTIF(BO4:BO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BP30" s="11">
+      <c r="BP30" s="17">
         <f>COUNTIF(BP4:BP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BQ30" s="11">
+      <c r="BQ30" s="17">
         <f>COUNTIF(BQ4:BQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BR30" s="11">
+      <c r="BR30" s="17">
         <f>COUNTIF(BR4:BR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BS30" s="11">
+      <c r="BS30" s="17">
         <f>COUNTIF(BS4:BS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BT30" s="11">
+      <c r="BT30" s="17">
         <f>COUNTIF(BT4:BT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BU30" s="11">
+      <c r="BU30" s="17">
         <f>COUNTIF(BU4:BU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BV30" s="11">
+      <c r="BV30" s="17">
         <f>COUNTIF(BV4:BV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BW30" s="11">
+      <c r="BW30" s="17">
         <f>COUNTIF(BW4:BW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BX30" s="11">
+      <c r="BX30" s="17">
         <f>COUNTIF(BX4:BX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BY30" s="11">
+      <c r="BY30" s="17">
         <f>COUNTIF(BY4:BY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BZ30" s="11">
+      <c r="BZ30" s="17">
         <f>COUNTIF(BZ4:BZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CA30" s="11">
+      <c r="CA30" s="17">
         <f>COUNTIF(CA4:CA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CB30" s="11">
+      <c r="CB30" s="17">
         <f>COUNTIF(CB4:CB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CC30" s="11">
+      <c r="CC30" s="17">
         <f>COUNTIF(CC4:CC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CD30" s="11">
+      <c r="CD30" s="17">
         <f>COUNTIF(CD4:CD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CE30" s="11">
+      <c r="CE30" s="17">
         <f>COUNTIF(CE4:CE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CF30" s="11">
+      <c r="CF30" s="17">
         <f>COUNTIF(CF4:CF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CG30" s="11">
+      <c r="CG30" s="17">
         <f>COUNTIF(CG4:CG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CH30" s="11">
+      <c r="CH30" s="17">
         <f>COUNTIF(CH4:CH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CI30" s="11">
+      <c r="CI30" s="17">
         <f>COUNTIF(CI4:CI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CJ30" s="11">
+      <c r="CJ30" s="17">
         <f>COUNTIF(CJ4:CJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CK30" s="11">
+      <c r="CK30" s="17">
         <f>COUNTIF(CK4:CK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CL30" s="11">
+      <c r="CL30" s="17">
         <f>COUNTIF(CL4:CL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CM30" s="11">
+      <c r="CM30" s="17">
         <f>COUNTIF(CM4:CM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CN30" s="11">
+      <c r="CN30" s="17">
         <f>COUNTIF(CN4:CN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CO30" s="11">
+      <c r="CO30" s="17">
         <f>COUNTIF(CO4:CO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CP30" s="11">
+      <c r="CP30" s="17">
         <f>COUNTIF(CP4:CP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CQ30" s="11">
+      <c r="CQ30" s="17">
         <f>COUNTIF(CQ4:CQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CR30" s="11">
+      <c r="CR30" s="17">
         <f>COUNTIF(CR4:CR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CS30" s="11">
+      <c r="CS30" s="17">
         <f>COUNTIF(CS4:CS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CT30" s="11">
+      <c r="CT30" s="17">
         <f>COUNTIF(CT4:CT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CU30" s="11">
+      <c r="CU30" s="17">
         <f>COUNTIF(CU4:CU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CV30" s="11">
+      <c r="CV30" s="17">
         <f>COUNTIF(CV4:CV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CW30" s="11">
+      <c r="CW30" s="17">
         <f>COUNTIF(CW4:CW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CX30" s="11">
+      <c r="CX30" s="17">
         <f>COUNTIF(CX4:CX29,"בסיס")</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>נשקייה בבסיס</t>
         </is>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",D4:D29,"בסיס")</f>
         <v/>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",E4:E29,"בסיס")</f>
         <v/>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",F4:F29,"בסיס")</f>
         <v/>
       </c>
-      <c r="G31" s="11">
+      <c r="G31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",G4:G29,"בסיס")</f>
         <v/>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",H4:H29,"בסיס")</f>
         <v/>
       </c>
-      <c r="I31" s="11">
+      <c r="I31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",I4:I29,"בסיס")</f>
         <v/>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",J4:J29,"בסיס")</f>
         <v/>
       </c>
-      <c r="K31" s="11">
+      <c r="K31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",K4:K29,"בסיס")</f>
         <v/>
       </c>
-      <c r="L31" s="11">
+      <c r="L31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",L4:L29,"בסיס")</f>
         <v/>
       </c>
-      <c r="M31" s="11">
+      <c r="M31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",M4:M29,"בסיס")</f>
         <v/>
       </c>
-      <c r="N31" s="11">
+      <c r="N31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",N4:N29,"בסיס")</f>
         <v/>
       </c>
-      <c r="O31" s="11">
+      <c r="O31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",O4:O29,"בסיס")</f>
         <v/>
       </c>
-      <c r="P31" s="11">
+      <c r="P31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",P4:P29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Q31" s="11">
+      <c r="Q31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",Q4:Q29,"בסיס")</f>
         <v/>
       </c>
-      <c r="R31" s="11">
+      <c r="R31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",R4:R29,"בסיס")</f>
         <v/>
       </c>
-      <c r="S31" s="11">
+      <c r="S31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",S4:S29,"בסיס")</f>
         <v/>
       </c>
-      <c r="T31" s="11">
+      <c r="T31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",T4:T29,"בסיס")</f>
         <v/>
       </c>
-      <c r="U31" s="11">
+      <c r="U31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",U4:U29,"בסיס")</f>
         <v/>
       </c>
-      <c r="V31" s="11">
+      <c r="V31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",V4:V29,"בסיס")</f>
         <v/>
       </c>
-      <c r="W31" s="11">
+      <c r="W31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",W4:W29,"בסיס")</f>
         <v/>
       </c>
-      <c r="X31" s="11">
+      <c r="X31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",X4:X29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Y31" s="11">
+      <c r="Y31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",Y4:Y29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Z31" s="11">
+      <c r="Z31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",Z4:Z29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AA31" s="11">
+      <c r="AA31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AA4:AA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AB31" s="11">
+      <c r="AB31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AB4:AB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AC31" s="11">
+      <c r="AC31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AC4:AC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AD31" s="11">
+      <c r="AD31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AD4:AD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AE31" s="11">
+      <c r="AE31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AE4:AE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AF31" s="11">
+      <c r="AF31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AF4:AF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AG31" s="11">
+      <c r="AG31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AG4:AG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AH31" s="11">
+      <c r="AH31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AH4:AH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AI31" s="11">
+      <c r="AI31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AI4:AI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AJ31" s="11">
+      <c r="AJ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AJ4:AJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AK31" s="11">
+      <c r="AK31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AK4:AK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AL31" s="11">
+      <c r="AL31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AL4:AL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AM31" s="11">
+      <c r="AM31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AM4:AM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AN31" s="11">
+      <c r="AN31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AN4:AN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AO31" s="11">
+      <c r="AO31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AO4:AO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AP31" s="11">
+      <c r="AP31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AP4:AP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AQ31" s="11">
+      <c r="AQ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AQ4:AQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AR31" s="11">
+      <c r="AR31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AR4:AR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AS31" s="11">
+      <c r="AS31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AS4:AS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AT31" s="11">
+      <c r="AT31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AT4:AT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AU31" s="11">
+      <c r="AU31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AU4:AU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AV31" s="11">
+      <c r="AV31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AV4:AV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AW31" s="11">
+      <c r="AW31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AW4:AW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AX31" s="11">
+      <c r="AX31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AX4:AX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AY31" s="11">
+      <c r="AY31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AY4:AY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AZ31" s="11">
+      <c r="AZ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",AZ4:AZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BA31" s="11">
+      <c r="BA31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BA4:BA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BB31" s="11">
+      <c r="BB31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BB4:BB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BC31" s="11">
+      <c r="BC31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BC4:BC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BD31" s="11">
+      <c r="BD31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BD4:BD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BE31" s="11">
+      <c r="BE31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BE4:BE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BF31" s="11">
+      <c r="BF31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BF4:BF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BG31" s="11">
+      <c r="BG31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BG4:BG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BH31" s="11">
+      <c r="BH31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BH4:BH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BI31" s="11">
+      <c r="BI31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BI4:BI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BJ31" s="11">
+      <c r="BJ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BJ4:BJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BK31" s="11">
+      <c r="BK31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BK4:BK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BL31" s="11">
+      <c r="BL31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BL4:BL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BM31" s="11">
+      <c r="BM31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BM4:BM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BN31" s="11">
+      <c r="BN31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BN4:BN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BO31" s="11">
+      <c r="BO31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BO4:BO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BP31" s="11">
+      <c r="BP31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BP4:BP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BQ31" s="11">
+      <c r="BQ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BQ4:BQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BR31" s="11">
+      <c r="BR31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BR4:BR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BS31" s="11">
+      <c r="BS31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BS4:BS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BT31" s="11">
+      <c r="BT31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BT4:BT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BU31" s="11">
+      <c r="BU31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BU4:BU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BV31" s="11">
+      <c r="BV31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BV4:BV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BW31" s="11">
+      <c r="BW31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BW4:BW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BX31" s="11">
+      <c r="BX31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BX4:BX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BY31" s="11">
+      <c r="BY31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BY4:BY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BZ31" s="11">
+      <c r="BZ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",BZ4:BZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CA31" s="11">
+      <c r="CA31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CA4:CA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CB31" s="11">
+      <c r="CB31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CB4:CB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CC31" s="11">
+      <c r="CC31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CC4:CC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CD31" s="11">
+      <c r="CD31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CD4:CD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CE31" s="11">
+      <c r="CE31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CE4:CE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CF31" s="11">
+      <c r="CF31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CF4:CF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CG31" s="11">
+      <c r="CG31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CG4:CG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CH31" s="11">
+      <c r="CH31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CH4:CH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CI31" s="11">
+      <c r="CI31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CI4:CI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CJ31" s="11">
+      <c r="CJ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CJ4:CJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CK31" s="11">
+      <c r="CK31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CK4:CK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CL31" s="11">
+      <c r="CL31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CL4:CL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CM31" s="11">
+      <c r="CM31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CM4:CM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CN31" s="11">
+      <c r="CN31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CN4:CN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CO31" s="11">
+      <c r="CO31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CO4:CO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CP31" s="11">
+      <c r="CP31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CP4:CP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CQ31" s="11">
+      <c r="CQ31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CQ4:CQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CR31" s="11">
+      <c r="CR31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CR4:CR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CS31" s="11">
+      <c r="CS31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CS4:CS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CT31" s="11">
+      <c r="CT31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CT4:CT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CU31" s="11">
+      <c r="CU31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CU4:CU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CV31" s="11">
+      <c r="CV31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CV4:CV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CW31" s="11">
+      <c r="CW31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CW4:CW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CX31" s="11">
+      <c r="CX31" s="17">
         <f>COUNTIFS($B$4:$B$29,"*נשקייה*",CX4:CX29,"בסיס")</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>אפסנאות בבסיס</t>
         </is>
       </c>
-      <c r="D32" s="11">
+      <c r="D32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",D4:D29,"בסיס")</f>
         <v/>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",E4:E29,"בסיס")</f>
         <v/>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",F4:F29,"בסיס")</f>
         <v/>
       </c>
-      <c r="G32" s="11">
+      <c r="G32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",G4:G29,"בסיס")</f>
         <v/>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",H4:H29,"בסיס")</f>
         <v/>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",I4:I29,"בסיס")</f>
         <v/>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",J4:J29,"בסיס")</f>
         <v/>
       </c>
-      <c r="K32" s="11">
+      <c r="K32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",K4:K29,"בסיס")</f>
         <v/>
       </c>
-      <c r="L32" s="11">
+      <c r="L32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",L4:L29,"בסיס")</f>
         <v/>
       </c>
-      <c r="M32" s="11">
+      <c r="M32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",M4:M29,"בסיס")</f>
         <v/>
       </c>
-      <c r="N32" s="11">
+      <c r="N32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",N4:N29,"בסיס")</f>
         <v/>
       </c>
-      <c r="O32" s="11">
+      <c r="O32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",O4:O29,"בסיס")</f>
         <v/>
       </c>
-      <c r="P32" s="11">
+      <c r="P32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",P4:P29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Q32" s="11">
+      <c r="Q32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",Q4:Q29,"בסיס")</f>
         <v/>
       </c>
-      <c r="R32" s="11">
+      <c r="R32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",R4:R29,"בסיס")</f>
         <v/>
       </c>
-      <c r="S32" s="11">
+      <c r="S32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",S4:S29,"בסיס")</f>
         <v/>
       </c>
-      <c r="T32" s="11">
+      <c r="T32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",T4:T29,"בסיס")</f>
         <v/>
       </c>
-      <c r="U32" s="11">
+      <c r="U32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",U4:U29,"בסיס")</f>
         <v/>
       </c>
-      <c r="V32" s="11">
+      <c r="V32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",V4:V29,"בסיס")</f>
         <v/>
       </c>
-      <c r="W32" s="11">
+      <c r="W32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",W4:W29,"בסיס")</f>
         <v/>
       </c>
-      <c r="X32" s="11">
+      <c r="X32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",X4:X29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Y32" s="11">
+      <c r="Y32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",Y4:Y29,"בסיס")</f>
         <v/>
       </c>
-      <c r="Z32" s="11">
+      <c r="Z32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",Z4:Z29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AA32" s="11">
+      <c r="AA32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AA4:AA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AB32" s="11">
+      <c r="AB32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AB4:AB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AC32" s="11">
+      <c r="AC32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AC4:AC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AD32" s="11">
+      <c r="AD32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AD4:AD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AE32" s="11">
+      <c r="AE32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AE4:AE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AF32" s="11">
+      <c r="AF32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AF4:AF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AG32" s="11">
+      <c r="AG32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AG4:AG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AH32" s="11">
+      <c r="AH32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AH4:AH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AI32" s="11">
+      <c r="AI32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AI4:AI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AJ32" s="11">
+      <c r="AJ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AJ4:AJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AK32" s="11">
+      <c r="AK32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AK4:AK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AL32" s="11">
+      <c r="AL32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AL4:AL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AM32" s="11">
+      <c r="AM32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AM4:AM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AN32" s="11">
+      <c r="AN32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AN4:AN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AO32" s="11">
+      <c r="AO32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AO4:AO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AP32" s="11">
+      <c r="AP32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AP4:AP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AQ32" s="11">
+      <c r="AQ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AQ4:AQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AR32" s="11">
+      <c r="AR32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AR4:AR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AS32" s="11">
+      <c r="AS32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AS4:AS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AT32" s="11">
+      <c r="AT32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AT4:AT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AU32" s="11">
+      <c r="AU32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AU4:AU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AV32" s="11">
+      <c r="AV32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AV4:AV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AW32" s="11">
+      <c r="AW32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AW4:AW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AX32" s="11">
+      <c r="AX32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AX4:AX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AY32" s="11">
+      <c r="AY32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AY4:AY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="AZ32" s="11">
+      <c r="AZ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",AZ4:AZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BA32" s="11">
+      <c r="BA32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BA4:BA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BB32" s="11">
+      <c r="BB32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BB4:BB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BC32" s="11">
+      <c r="BC32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BC4:BC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BD32" s="11">
+      <c r="BD32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BD4:BD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BE32" s="11">
+      <c r="BE32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BE4:BE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BF32" s="11">
+      <c r="BF32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BF4:BF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BG32" s="11">
+      <c r="BG32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BG4:BG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BH32" s="11">
+      <c r="BH32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BH4:BH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BI32" s="11">
+      <c r="BI32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BI4:BI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BJ32" s="11">
+      <c r="BJ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BJ4:BJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BK32" s="11">
+      <c r="BK32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BK4:BK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BL32" s="11">
+      <c r="BL32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BL4:BL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BM32" s="11">
+      <c r="BM32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BM4:BM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BN32" s="11">
+      <c r="BN32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BN4:BN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BO32" s="11">
+      <c r="BO32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BO4:BO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BP32" s="11">
+      <c r="BP32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BP4:BP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BQ32" s="11">
+      <c r="BQ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BQ4:BQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BR32" s="11">
+      <c r="BR32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BR4:BR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BS32" s="11">
+      <c r="BS32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BS4:BS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BT32" s="11">
+      <c r="BT32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BT4:BT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BU32" s="11">
+      <c r="BU32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BU4:BU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BV32" s="11">
+      <c r="BV32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BV4:BV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BW32" s="11">
+      <c r="BW32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BW4:BW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BX32" s="11">
+      <c r="BX32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BX4:BX29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BY32" s="11">
+      <c r="BY32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BY4:BY29,"בסיס")</f>
         <v/>
       </c>
-      <c r="BZ32" s="11">
+      <c r="BZ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",BZ4:BZ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CA32" s="11">
+      <c r="CA32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CA4:CA29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CB32" s="11">
+      <c r="CB32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CB4:CB29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CC32" s="11">
+      <c r="CC32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CC4:CC29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CD32" s="11">
+      <c r="CD32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CD4:CD29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CE32" s="11">
+      <c r="CE32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CE4:CE29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CF32" s="11">
+      <c r="CF32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CF4:CF29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CG32" s="11">
+      <c r="CG32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CG4:CG29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CH32" s="11">
+      <c r="CH32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CH4:CH29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CI32" s="11">
+      <c r="CI32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CI4:CI29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CJ32" s="11">
+      <c r="CJ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CJ4:CJ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CK32" s="11">
+      <c r="CK32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CK4:CK29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CL32" s="11">
+      <c r="CL32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CL4:CL29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CM32" s="11">
+      <c r="CM32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CM4:CM29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CN32" s="11">
+      <c r="CN32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CN4:CN29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CO32" s="11">
+      <c r="CO32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CO4:CO29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CP32" s="11">
+      <c r="CP32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CP4:CP29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CQ32" s="11">
+      <c r="CQ32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CQ4:CQ29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CR32" s="11">
+      <c r="CR32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CR4:CR29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CS32" s="11">
+      <c r="CS32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CS4:CS29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CT32" s="11">
+      <c r="CT32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CT4:CT29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CU32" s="11">
+      <c r="CU32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CU4:CU29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CV32" s="11">
+      <c r="CV32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CV4:CV29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CW32" s="11">
+      <c r="CW32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CW4:CW29,"בסיס")</f>
         <v/>
       </c>
-      <c r="CX32" s="11">
+      <c r="CX32" s="17">
         <f>COUNTIFS($B$4:$B$29,"*אפסנאות*",CX4:CX29,"בסיס")</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>סה"כ בבית</t>
         </is>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="17">
         <f>COUNTIF(D4:D29,"בית")</f>
         <v/>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="17">
         <f>COUNTIF(E4:E29,"בית")</f>
         <v/>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="17">
         <f>COUNTIF(F4:F29,"בית")</f>
         <v/>
       </c>
-      <c r="G33" s="11">
+      <c r="G33" s="17">
         <f>COUNTIF(G4:G29,"בית")</f>
         <v/>
       </c>
-      <c r="H33" s="11">
+      <c r="H33" s="17">
         <f>COUNTIF(H4:H29,"בית")</f>
         <v/>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="17">
         <f>COUNTIF(I4:I29,"בית")</f>
         <v/>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="17">
         <f>COUNTIF(J4:J29,"בית")</f>
         <v/>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="17">
         <f>COUNTIF(K4:K29,"בית")</f>
         <v/>
       </c>
-      <c r="L33" s="11">
+      <c r="L33" s="17">
         <f>COUNTIF(L4:L29,"בית")</f>
         <v/>
       </c>
-      <c r="M33" s="11">
+      <c r="M33" s="17">
         <f>COUNTIF(M4:M29,"בית")</f>
         <v/>
       </c>
-      <c r="N33" s="11">
+      <c r="N33" s="17">
         <f>COUNTIF(N4:N29,"בית")</f>
         <v/>
       </c>
-      <c r="O33" s="11">
+      <c r="O33" s="17">
         <f>COUNTIF(O4:O29,"בית")</f>
         <v/>
       </c>
-      <c r="P33" s="11">
+      <c r="P33" s="17">
         <f>COUNTIF(P4:P29,"בית")</f>
         <v/>
       </c>
-      <c r="Q33" s="11">
+      <c r="Q33" s="17">
         <f>COUNTIF(Q4:Q29,"בית")</f>
         <v/>
       </c>
-      <c r="R33" s="11">
+      <c r="R33" s="17">
         <f>COUNTIF(R4:R29,"בית")</f>
         <v/>
       </c>
-      <c r="S33" s="11">
+      <c r="S33" s="17">
         <f>COUNTIF(S4:S29,"בית")</f>
         <v/>
       </c>
-      <c r="T33" s="11">
+      <c r="T33" s="17">
         <f>COUNTIF(T4:T29,"בית")</f>
         <v/>
       </c>
-      <c r="U33" s="11">
+      <c r="U33" s="17">
         <f>COUNTIF(U4:U29,"בית")</f>
         <v/>
       </c>
-      <c r="V33" s="11">
+      <c r="V33" s="17">
         <f>COUNTIF(V4:V29,"בית")</f>
         <v/>
       </c>
-      <c r="W33" s="11">
+      <c r="W33" s="17">
         <f>COUNTIF(W4:W29,"בית")</f>
         <v/>
       </c>
-      <c r="X33" s="11">
+      <c r="X33" s="17">
         <f>COUNTIF(X4:X29,"בית")</f>
         <v/>
       </c>
-      <c r="Y33" s="11">
+      <c r="Y33" s="17">
         <f>COUNTIF(Y4:Y29,"בית")</f>
         <v/>
       </c>
-      <c r="Z33" s="11">
+      <c r="Z33" s="17">
         <f>COUNTIF(Z4:Z29,"בית")</f>
         <v/>
       </c>
-      <c r="AA33" s="11">
+      <c r="AA33" s="17">
         <f>COUNTIF(AA4:AA29,"בית")</f>
         <v/>
       </c>
-      <c r="AB33" s="11">
+      <c r="AB33" s="17">
         <f>COUNTIF(AB4:AB29,"בית")</f>
         <v/>
       </c>
-      <c r="AC33" s="11">
+      <c r="AC33" s="17">
         <f>COUNTIF(AC4:AC29,"בית")</f>
         <v/>
       </c>
-      <c r="AD33" s="11">
+      <c r="AD33" s="17">
         <f>COUNTIF(AD4:AD29,"בית")</f>
         <v/>
       </c>
-      <c r="AE33" s="11">
+      <c r="AE33" s="17">
         <f>COUNTIF(AE4:AE29,"בית")</f>
         <v/>
       </c>
-      <c r="AF33" s="11">
+      <c r="AF33" s="17">
         <f>COUNTIF(AF4:AF29,"בית")</f>
         <v/>
       </c>
-      <c r="AG33" s="11">
+      <c r="AG33" s="17">
         <f>COUNTIF(AG4:AG29,"בית")</f>
         <v/>
       </c>
-      <c r="AH33" s="11">
+      <c r="AH33" s="17">
         <f>COUNTIF(AH4:AH29,"בית")</f>
         <v/>
       </c>
-      <c r="AI33" s="11">
+      <c r="AI33" s="17">
         <f>COUNTIF(AI4:AI29,"בית")</f>
         <v/>
       </c>
-      <c r="AJ33" s="11">
+      <c r="AJ33" s="17">
         <f>COUNTIF(AJ4:AJ29,"בית")</f>
         <v/>
       </c>
-      <c r="AK33" s="11">
+      <c r="AK33" s="17">
         <f>COUNTIF(AK4:AK29,"בית")</f>
         <v/>
       </c>
-      <c r="AL33" s="11">
+      <c r="AL33" s="17">
         <f>COUNTIF(AL4:AL29,"בית")</f>
         <v/>
       </c>
-      <c r="AM33" s="11">
+      <c r="AM33" s="17">
         <f>COUNTIF(AM4:AM29,"בית")</f>
         <v/>
       </c>
-      <c r="AN33" s="11">
+      <c r="AN33" s="17">
         <f>COUNTIF(AN4:AN29,"בית")</f>
         <v/>
       </c>
-      <c r="AO33" s="11">
+      <c r="AO33" s="17">
         <f>COUNTIF(AO4:AO29,"בית")</f>
         <v/>
       </c>
-      <c r="AP33" s="11">
+      <c r="AP33" s="17">
         <f>COUNTIF(AP4:AP29,"בית")</f>
         <v/>
       </c>
-      <c r="AQ33" s="11">
+      <c r="AQ33" s="17">
         <f>COUNTIF(AQ4:AQ29,"בית")</f>
         <v/>
       </c>
-      <c r="AR33" s="11">
+      <c r="AR33" s="17">
         <f>COUNTIF(AR4:AR29,"בית")</f>
         <v/>
       </c>
-      <c r="AS33" s="11">
+      <c r="AS33" s="17">
         <f>COUNTIF(AS4:AS29,"בית")</f>
         <v/>
       </c>
-      <c r="AT33" s="11">
+      <c r="AT33" s="17">
         <f>COUNTIF(AT4:AT29,"בית")</f>
         <v/>
       </c>
-      <c r="AU33" s="11">
+      <c r="AU33" s="17">
         <f>COUNTIF(AU4:AU29,"בית")</f>
         <v/>
       </c>
-      <c r="AV33" s="11">
+      <c r="AV33" s="17">
         <f>COUNTIF(AV4:AV29,"בית")</f>
         <v/>
       </c>
-      <c r="AW33" s="11">
+      <c r="AW33" s="17">
         <f>COUNTIF(AW4:AW29,"בית")</f>
         <v/>
       </c>
-      <c r="AX33" s="11">
+      <c r="AX33" s="17">
         <f>COUNTIF(AX4:AX29,"בית")</f>
         <v/>
       </c>
-      <c r="AY33" s="11">
+      <c r="AY33" s="17">
         <f>COUNTIF(AY4:AY29,"בית")</f>
         <v/>
       </c>
-      <c r="AZ33" s="11">
+      <c r="AZ33" s="17">
         <f>COUNTIF(AZ4:AZ29,"בית")</f>
         <v/>
       </c>
-      <c r="BA33" s="11">
+      <c r="BA33" s="17">
         <f>COUNTIF(BA4:BA29,"בית")</f>
         <v/>
       </c>
-      <c r="BB33" s="11">
+      <c r="BB33" s="17">
         <f>COUNTIF(BB4:BB29,"בית")</f>
         <v/>
       </c>
-      <c r="BC33" s="11">
+      <c r="BC33" s="17">
         <f>COUNTIF(BC4:BC29,"בית")</f>
         <v/>
       </c>
-      <c r="BD33" s="11">
+      <c r="BD33" s="17">
         <f>COUNTIF(BD4:BD29,"בית")</f>
         <v/>
       </c>
-      <c r="BE33" s="11">
+      <c r="BE33" s="17">
         <f>COUNTIF(BE4:BE29,"בית")</f>
         <v/>
       </c>
-      <c r="BF33" s="11">
+      <c r="BF33" s="17">
         <f>COUNTIF(BF4:BF29,"בית")</f>
         <v/>
       </c>
-      <c r="BG33" s="11">
+      <c r="BG33" s="17">
         <f>COUNTIF(BG4:BG29,"בית")</f>
         <v/>
       </c>
-      <c r="BH33" s="11">
+      <c r="BH33" s="17">
         <f>COUNTIF(BH4:BH29,"בית")</f>
         <v/>
       </c>
-      <c r="BI33" s="11">
+      <c r="BI33" s="17">
         <f>COUNTIF(BI4:BI29,"בית")</f>
         <v/>
       </c>
-      <c r="BJ33" s="11">
+      <c r="BJ33" s="17">
         <f>COUNTIF(BJ4:BJ29,"בית")</f>
         <v/>
       </c>
-      <c r="BK33" s="11">
+      <c r="BK33" s="17">
         <f>COUNTIF(BK4:BK29,"בית")</f>
         <v/>
       </c>
-      <c r="BL33" s="11">
+      <c r="BL33" s="17">
         <f>COUNTIF(BL4:BL29,"בית")</f>
         <v/>
       </c>
-      <c r="BM33" s="11">
+      <c r="BM33" s="17">
         <f>COUNTIF(BM4:BM29,"בית")</f>
         <v/>
       </c>
-      <c r="BN33" s="11">
+      <c r="BN33" s="17">
         <f>COUNTIF(BN4:BN29,"בית")</f>
         <v/>
       </c>
-      <c r="BO33" s="11">
+      <c r="BO33" s="17">
         <f>COUNTIF(BO4:BO29,"בית")</f>
         <v/>
       </c>
-      <c r="BP33" s="11">
+      <c r="BP33" s="17">
         <f>COUNTIF(BP4:BP29,"בית")</f>
         <v/>
       </c>
-      <c r="BQ33" s="11">
+      <c r="BQ33" s="17">
         <f>COUNTIF(BQ4:BQ29,"בית")</f>
         <v/>
       </c>
-      <c r="BR33" s="11">
+      <c r="BR33" s="17">
         <f>COUNTIF(BR4:BR29,"בית")</f>
         <v/>
       </c>
-      <c r="BS33" s="11">
+      <c r="BS33" s="17">
         <f>COUNTIF(BS4:BS29,"בית")</f>
         <v/>
       </c>
-      <c r="BT33" s="11">
+      <c r="BT33" s="17">
         <f>COUNTIF(BT4:BT29,"בית")</f>
         <v/>
       </c>
-      <c r="BU33" s="11">
+      <c r="BU33" s="17">
         <f>COUNTIF(BU4:BU29,"בית")</f>
         <v/>
       </c>
-      <c r="BV33" s="11">
+      <c r="BV33" s="17">
         <f>COUNTIF(BV4:BV29,"בית")</f>
         <v/>
       </c>
-      <c r="BW33" s="11">
+      <c r="BW33" s="17">
         <f>COUNTIF(BW4:BW29,"בית")</f>
         <v/>
       </c>
-      <c r="BX33" s="11">
+      <c r="BX33" s="17">
         <f>COUNTIF(BX4:BX29,"בית")</f>
         <v/>
       </c>
-      <c r="BY33" s="11">
+      <c r="BY33" s="17">
         <f>COUNTIF(BY4:BY29,"בית")</f>
         <v/>
       </c>
-      <c r="BZ33" s="11">
+      <c r="BZ33" s="17">
         <f>COUNTIF(BZ4:BZ29,"בית")</f>
         <v/>
       </c>
-      <c r="CA33" s="11">
+      <c r="CA33" s="17">
         <f>COUNTIF(CA4:CA29,"בית")</f>
         <v/>
       </c>
-      <c r="CB33" s="11">
+      <c r="CB33" s="17">
         <f>COUNTIF(CB4:CB29,"בית")</f>
         <v/>
       </c>
-      <c r="CC33" s="11">
+      <c r="CC33" s="17">
         <f>COUNTIF(CC4:CC29,"בית")</f>
         <v/>
       </c>
-      <c r="CD33" s="11">
+      <c r="CD33" s="17">
         <f>COUNTIF(CD4:CD29,"בית")</f>
         <v/>
       </c>
-      <c r="CE33" s="11">
+      <c r="CE33" s="17">
         <f>COUNTIF(CE4:CE29,"בית")</f>
         <v/>
       </c>
-      <c r="CF33" s="11">
+      <c r="CF33" s="17">
         <f>COUNTIF(CF4:CF29,"בית")</f>
         <v/>
       </c>
-      <c r="CG33" s="11">
+      <c r="CG33" s="17">
         <f>COUNTIF(CG4:CG29,"בית")</f>
         <v/>
       </c>
-      <c r="CH33" s="11">
+      <c r="CH33" s="17">
         <f>COUNTIF(CH4:CH29,"בית")</f>
         <v/>
       </c>
-      <c r="CI33" s="11">
+      <c r="CI33" s="17">
         <f>COUNTIF(CI4:CI29,"בית")</f>
         <v/>
       </c>
-      <c r="CJ33" s="11">
+      <c r="CJ33" s="17">
         <f>COUNTIF(CJ4:CJ29,"בית")</f>
         <v/>
       </c>
-      <c r="CK33" s="11">
+      <c r="CK33" s="17">
         <f>COUNTIF(CK4:CK29,"בית")</f>
         <v/>
       </c>
-      <c r="CL33" s="11">
+      <c r="CL33" s="17">
         <f>COUNTIF(CL4:CL29,"בית")</f>
         <v/>
       </c>
-      <c r="CM33" s="11">
+      <c r="CM33" s="17">
         <f>COUNTIF(CM4:CM29,"בית")</f>
         <v/>
       </c>
-      <c r="CN33" s="11">
+      <c r="CN33" s="17">
         <f>COUNTIF(CN4:CN29,"בית")</f>
         <v/>
       </c>
-      <c r="CO33" s="11">
+      <c r="CO33" s="17">
         <f>COUNTIF(CO4:CO29,"בית")</f>
         <v/>
       </c>
-      <c r="CP33" s="11">
+      <c r="CP33" s="17">
         <f>COUNTIF(CP4:CP29,"בית")</f>
         <v/>
       </c>
-      <c r="CQ33" s="11">
+      <c r="CQ33" s="17">
         <f>COUNTIF(CQ4:CQ29,"בית")</f>
         <v/>
       </c>
-      <c r="CR33" s="11">
+      <c r="CR33" s="17">
         <f>COUNTIF(CR4:CR29,"בית")</f>
         <v/>
       </c>
-      <c r="CS33" s="11">
+      <c r="CS33" s="17">
         <f>COUNTIF(CS4:CS29,"בית")</f>
         <v/>
       </c>
-      <c r="CT33" s="11">
+      <c r="CT33" s="17">
         <f>COUNTIF(CT4:CT29,"בית")</f>
         <v/>
       </c>
-      <c r="CU33" s="11">
+      <c r="CU33" s="17">
         <f>COUNTIF(CU4:CU29,"בית")</f>
         <v/>
       </c>
-      <c r="CV33" s="11">
+      <c r="CV33" s="17">
         <f>COUNTIF(CV4:CV29,"בית")</f>
         <v/>
       </c>
-      <c r="CW33" s="11">
+      <c r="CW33" s="17">
         <f>COUNTIF(CW4:CW29,"בית")</f>
         <v/>
       </c>
-      <c r="CX33" s="11">
+      <c r="CX33" s="17">
         <f>COUNTIF(CX4:CX29,"בית")</f>
         <v/>
       </c>
@@ -6939,14 +6993,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>הגדרות מצבה (ניתן לעריכה):</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>מינימום בבסיס</t>
         </is>
@@ -6956,7 +7010,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>מינימום נשקייה</t>
         </is>
@@ -6966,7 +7020,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>מינימום אפסנאות</t>
         </is>
@@ -7057,107 +7111,107 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>מקרא - שבצק יציאות</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>כותרת תאריך:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="n"/>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="A4" s="21" t="n"/>
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>שבת / ערב שבת</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>חג</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>סטטוס תא:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="A7" s="24" t="n"/>
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>בסיס</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="A8" s="25" t="n"/>
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>בית</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="A9" s="26" t="n"/>
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>חופשה</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="n"/>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="A10" s="27" t="n"/>
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>גימלים</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="A11" s="28" t="n"/>
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>קורס</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="A12" s="29" t="n"/>
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>ת״ש</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>התראות:</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="n"/>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="A14" s="30" t="n"/>
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>מתחת לסף מצבה (אדום אוטומטי)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>ספי המצבה נקבעים בגיליון השבצק בבלוק "הגדרות מצבה".</t>
         </is>
@@ -7235,10 +7289,10 @@
           <t>קלג</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -7251,10 +7305,10 @@
           <t>סמל נשקייה</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -7267,10 +7321,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -7283,10 +7337,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -7299,10 +7353,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -7315,10 +7369,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -7331,10 +7385,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -7347,10 +7401,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -7363,10 +7417,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -7379,10 +7433,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -7395,10 +7449,10 @@
           <t>סמל אפסנאות</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -7411,10 +7465,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -7427,10 +7481,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -7443,10 +7497,10 @@
           <t>נשקייה-רחפנים</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -7455,10 +7509,10 @@
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -7467,10 +7521,10 @@
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -7483,10 +7537,10 @@
           <t>נשקייה</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -7499,10 +7553,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -7515,10 +7569,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -7527,10 +7581,10 @@
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -7543,10 +7597,10 @@
           <t>אפסנאות</t>
         </is>
       </c>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -7555,10 +7609,10 @@
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -7567,10 +7621,10 @@
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -7579,10 +7633,10 @@
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -7591,10 +7645,10 @@
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
-      <c r="F27" s="9" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -7603,29 +7657,29 @@
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>סה"כ שוחחו:</t>
         </is>
       </c>
-      <c r="B30" s="25">
+      <c r="B30" s="31">
         <f>COUNTIF(C3:C28,"כן")</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>נותרו לשיחה:</t>
         </is>
       </c>
-      <c r="B31" s="25">
+      <c r="B31" s="31">
         <f>COUNTIF(C3:C28,"לא")</f>
         <v/>
       </c>

</xml_diff>